<commit_message>
feat(km19): tính W6, W7, W9 Mố M2 mà bản vẽ tr.40 ghi 0 kg (quyết định chủ dự án)
- Chủ dự án chọn 11/10/2026: tính các thanh có dài và số lượng nhưng bản vẽ ghi 0 kg (237,05 kg =
  51,50 + 48,84 + 136,71). Cấu hình 'tinh_dong_ban_ve_ghi_0' cho hạng mục; số cộng thêm tính tự động
  từ dài × SL × kg/m của các dòng đó (zero_weight_rows_kg), không gõ tay.
- BBS: tổng đối chiếu Mố M2 = 19.885,78 kg; BBS 19.876,96 (lệch −8,8 kg do quy ước kg/m) → khớp.
  Các dòng thép BBS không đổi nên bộ file cắt thép không cần sinh lại.
- Dự toán/03a: thép mố M2 = 19,64873 + 0,23705 t; G_XD 26.781.712.774 đ.
- Sửa lỗi công thức F dự toán cắt còn 6 chữ số có nghĩa (vd. 16,1778 thay vì 16,17783).
- Harness: bbs_theo_hang_muc_vs_ban_ve_tham_dinh ĐẠT 15/15 hạng mục; còn 2 ca chưa đối chiếu được
  (03a đã ký, dự toán đã duyệt — chưa có file).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_013xu17UUNVqCoEvpVUxkPSc
</commit_message>
<xml_diff>
--- a/examples/HO_SO_CAU_KM19_529/02_XUONG_TIEN_CHE_COT_THEP/04_Thong_Ke_Thep_Chi_Tiet_BBS_396_Dong.xlsx
+++ b/examples/HO_SO_CAU_KM19_529/02_XUONG_TIEN_CHE_COT_THEP/04_Thong_Ke_Thep_Chi_Tiet_BBS_396_Dong.xlsx
@@ -4805,7 +4805,7 @@
       </c>
       <c r="R63" s="5" t="inlineStr">
         <is>
-          <t>Thay theo tr.40 (BBS cũ 19.981,23 kg, bản vẽ 19.648,73 kg)</t>
+          <t>Thay theo tr.40 (BBS cũ 19.981,23 kg, bản vẽ 19.885,78 kg)</t>
         </is>
       </c>
     </row>
@@ -4881,7 +4881,7 @@
       </c>
       <c r="R64" s="5" t="inlineStr">
         <is>
-          <t>Thay theo tr.40 (BBS cũ 19.981,23 kg, bản vẽ 19.648,73 kg)</t>
+          <t>Thay theo tr.40 (BBS cũ 19.981,23 kg, bản vẽ 19.885,78 kg)</t>
         </is>
       </c>
     </row>
@@ -4957,7 +4957,7 @@
       </c>
       <c r="R65" s="5" t="inlineStr">
         <is>
-          <t>Thay theo tr.40 (BBS cũ 19.981,23 kg, bản vẽ 19.648,73 kg)</t>
+          <t>Thay theo tr.40 (BBS cũ 19.981,23 kg, bản vẽ 19.885,78 kg)</t>
         </is>
       </c>
     </row>
@@ -5033,7 +5033,7 @@
       </c>
       <c r="R66" s="5" t="inlineStr">
         <is>
-          <t>Thay theo tr.40 (BBS cũ 19.981,23 kg, bản vẽ 19.648,73 kg)</t>
+          <t>Thay theo tr.40 (BBS cũ 19.981,23 kg, bản vẽ 19.885,78 kg)</t>
         </is>
       </c>
     </row>
@@ -5109,7 +5109,7 @@
       </c>
       <c r="R67" s="5" t="inlineStr">
         <is>
-          <t>Thay theo tr.40 (BBS cũ 19.981,23 kg, bản vẽ 19.648,73 kg)</t>
+          <t>Thay theo tr.40 (BBS cũ 19.981,23 kg, bản vẽ 19.885,78 kg)</t>
         </is>
       </c>
     </row>
@@ -5185,7 +5185,7 @@
       </c>
       <c r="R68" s="5" t="inlineStr">
         <is>
-          <t>Thay theo tr.40 (BBS cũ 19.981,23 kg, bản vẽ 19.648,73 kg)</t>
+          <t>Thay theo tr.40 (BBS cũ 19.981,23 kg, bản vẽ 19.885,78 kg)</t>
         </is>
       </c>
     </row>
@@ -5261,7 +5261,7 @@
       </c>
       <c r="R69" s="5" t="inlineStr">
         <is>
-          <t>Thay theo tr.40 (BBS cũ 19.981,23 kg, bản vẽ 19.648,73 kg)</t>
+          <t>Thay theo tr.40 (BBS cũ 19.981,23 kg, bản vẽ 19.885,78 kg)</t>
         </is>
       </c>
     </row>
@@ -5337,7 +5337,7 @@
       </c>
       <c r="R70" s="5" t="inlineStr">
         <is>
-          <t>Thay theo tr.40 (BBS cũ 19.981,23 kg, bản vẽ 19.648,73 kg)</t>
+          <t>Thay theo tr.40 (BBS cũ 19.981,23 kg, bản vẽ 19.885,78 kg)</t>
         </is>
       </c>
     </row>
@@ -5413,7 +5413,7 @@
       </c>
       <c r="R71" s="5" t="inlineStr">
         <is>
-          <t>Thay theo tr.40 (BBS cũ 19.981,23 kg, bản vẽ 19.648,73 kg)</t>
+          <t>Thay theo tr.40 (BBS cũ 19.981,23 kg, bản vẽ 19.885,78 kg)</t>
         </is>
       </c>
     </row>
@@ -5489,7 +5489,7 @@
       </c>
       <c r="R72" s="5" t="inlineStr">
         <is>
-          <t>Thay theo tr.40 (BBS cũ 19.981,23 kg, bản vẽ 19.648,73 kg)</t>
+          <t>Thay theo tr.40 (BBS cũ 19.981,23 kg, bản vẽ 19.885,78 kg)</t>
         </is>
       </c>
     </row>
@@ -5565,7 +5565,7 @@
       </c>
       <c r="R73" s="5" t="inlineStr">
         <is>
-          <t>Thay theo tr.40 (BBS cũ 19.981,23 kg, bản vẽ 19.648,73 kg)</t>
+          <t>Thay theo tr.40 (BBS cũ 19.981,23 kg, bản vẽ 19.885,78 kg)</t>
         </is>
       </c>
     </row>
@@ -5641,7 +5641,7 @@
       </c>
       <c r="R74" s="5" t="inlineStr">
         <is>
-          <t>Thay theo tr.40 (BBS cũ 19.981,23 kg, bản vẽ 19.648,73 kg)</t>
+          <t>Thay theo tr.40 (BBS cũ 19.981,23 kg, bản vẽ 19.885,78 kg)</t>
         </is>
       </c>
     </row>
@@ -5717,7 +5717,7 @@
       </c>
       <c r="R75" s="5" t="inlineStr">
         <is>
-          <t>Thay theo tr.40 (BBS cũ 19.981,23 kg, bản vẽ 19.648,73 kg)</t>
+          <t>Thay theo tr.40 (BBS cũ 19.981,23 kg, bản vẽ 19.885,78 kg)</t>
         </is>
       </c>
     </row>
@@ -5793,7 +5793,7 @@
       </c>
       <c r="R76" s="5" t="inlineStr">
         <is>
-          <t>Thay theo tr.40 (BBS cũ 19.981,23 kg, bản vẽ 19.648,73 kg)</t>
+          <t>Thay theo tr.40 (BBS cũ 19.981,23 kg, bản vẽ 19.885,78 kg)</t>
         </is>
       </c>
     </row>
@@ -5869,7 +5869,7 @@
       </c>
       <c r="R77" s="5" t="inlineStr">
         <is>
-          <t>Thay theo tr.40 (BBS cũ 19.981,23 kg, bản vẽ 19.648,73 kg)</t>
+          <t>Thay theo tr.40 (BBS cũ 19.981,23 kg, bản vẽ 19.885,78 kg)</t>
         </is>
       </c>
     </row>
@@ -5945,7 +5945,7 @@
       </c>
       <c r="R78" s="5" t="inlineStr">
         <is>
-          <t>Thay theo tr.40 (BBS cũ 19.981,23 kg, bản vẽ 19.648,73 kg)</t>
+          <t>Thay theo tr.40 (BBS cũ 19.981,23 kg, bản vẽ 19.885,78 kg)</t>
         </is>
       </c>
     </row>
@@ -6021,7 +6021,7 @@
       </c>
       <c r="R79" s="5" t="inlineStr">
         <is>
-          <t>Thay theo tr.40 (BBS cũ 19.981,23 kg, bản vẽ 19.648,73 kg)</t>
+          <t>Thay theo tr.40 (BBS cũ 19.981,23 kg, bản vẽ 19.885,78 kg)</t>
         </is>
       </c>
     </row>
@@ -6097,7 +6097,7 @@
       </c>
       <c r="R80" s="5" t="inlineStr">
         <is>
-          <t>Thay theo tr.40 (BBS cũ 19.981,23 kg, bản vẽ 19.648,73 kg)</t>
+          <t>Thay theo tr.40 (BBS cũ 19.981,23 kg, bản vẽ 19.885,78 kg)</t>
         </is>
       </c>
     </row>
@@ -6173,7 +6173,7 @@
       </c>
       <c r="R81" s="5" t="inlineStr">
         <is>
-          <t>Thay theo tr.40 (BBS cũ 19.981,23 kg, bản vẽ 19.648,73 kg)</t>
+          <t>Thay theo tr.40 (BBS cũ 19.981,23 kg, bản vẽ 19.885,78 kg)</t>
         </is>
       </c>
     </row>
@@ -6249,7 +6249,7 @@
       </c>
       <c r="R82" s="5" t="inlineStr">
         <is>
-          <t>Thay theo tr.40 (BBS cũ 19.981,23 kg, bản vẽ 19.648,73 kg)</t>
+          <t>Thay theo tr.40 (BBS cũ 19.981,23 kg, bản vẽ 19.885,78 kg)</t>
         </is>
       </c>
     </row>
@@ -6325,7 +6325,7 @@
       </c>
       <c r="R83" s="5" t="inlineStr">
         <is>
-          <t>Thay theo tr.40 (BBS cũ 19.981,23 kg, bản vẽ 19.648,73 kg)</t>
+          <t>Thay theo tr.40 (BBS cũ 19.981,23 kg, bản vẽ 19.885,78 kg)</t>
         </is>
       </c>
     </row>
@@ -6401,7 +6401,7 @@
       </c>
       <c r="R84" s="5" t="inlineStr">
         <is>
-          <t>Thay theo tr.40 (BBS cũ 19.981,23 kg, bản vẽ 19.648,73 kg)</t>
+          <t>Thay theo tr.40 (BBS cũ 19.981,23 kg, bản vẽ 19.885,78 kg)</t>
         </is>
       </c>
     </row>
@@ -6477,7 +6477,7 @@
       </c>
       <c r="R85" s="5" t="inlineStr">
         <is>
-          <t>Thay theo tr.40 (BBS cũ 19.981,23 kg, bản vẽ 19.648,73 kg)</t>
+          <t>Thay theo tr.40 (BBS cũ 19.981,23 kg, bản vẽ 19.885,78 kg)</t>
         </is>
       </c>
     </row>
@@ -6553,7 +6553,7 @@
       </c>
       <c r="R86" s="5" t="inlineStr">
         <is>
-          <t>Thay theo tr.40 (BBS cũ 19.981,23 kg, bản vẽ 19.648,73 kg)</t>
+          <t>Thay theo tr.40 (BBS cũ 19.981,23 kg, bản vẽ 19.885,78 kg)</t>
         </is>
       </c>
     </row>
@@ -6629,7 +6629,7 @@
       </c>
       <c r="R87" s="5" t="inlineStr">
         <is>
-          <t>Thay theo tr.40 (BBS cũ 19.981,23 kg, bản vẽ 19.648,73 kg)</t>
+          <t>Thay theo tr.40 (BBS cũ 19.981,23 kg, bản vẽ 19.885,78 kg)</t>
         </is>
       </c>
     </row>
@@ -6705,7 +6705,7 @@
       </c>
       <c r="R88" s="5" t="inlineStr">
         <is>
-          <t>Thay theo tr.40 (BBS cũ 19.981,23 kg, bản vẽ 19.648,73 kg)</t>
+          <t>Thay theo tr.40 (BBS cũ 19.981,23 kg, bản vẽ 19.885,78 kg)</t>
         </is>
       </c>
     </row>
@@ -6781,7 +6781,7 @@
       </c>
       <c r="R89" s="5" t="inlineStr">
         <is>
-          <t>Thay theo tr.40 (BBS cũ 19.981,23 kg, bản vẽ 19.648,73 kg)</t>
+          <t>Thay theo tr.40 (BBS cũ 19.981,23 kg, bản vẽ 19.885,78 kg)</t>
         </is>
       </c>
     </row>
@@ -6857,7 +6857,7 @@
       </c>
       <c r="R90" s="5" t="inlineStr">
         <is>
-          <t>Thay theo tr.40 (BBS cũ 19.981,23 kg, bản vẽ 19.648,73 kg)</t>
+          <t>Thay theo tr.40 (BBS cũ 19.981,23 kg, bản vẽ 19.885,78 kg)</t>
         </is>
       </c>
     </row>
@@ -6933,7 +6933,7 @@
       </c>
       <c r="R91" s="5" t="inlineStr">
         <is>
-          <t>Thay theo tr.40 (BBS cũ 19.981,23 kg, bản vẽ 19.648,73 kg)</t>
+          <t>Thay theo tr.40 (BBS cũ 19.981,23 kg, bản vẽ 19.885,78 kg)</t>
         </is>
       </c>
     </row>
@@ -7009,7 +7009,7 @@
       </c>
       <c r="R92" s="5" t="inlineStr">
         <is>
-          <t>Thay theo tr.40 (BBS cũ 19.981,23 kg, bản vẽ 19.648,73 kg)</t>
+          <t>Thay theo tr.40 (BBS cũ 19.981,23 kg, bản vẽ 19.885,78 kg)</t>
         </is>
       </c>
     </row>
@@ -7085,7 +7085,7 @@
       </c>
       <c r="R93" s="5" t="inlineStr">
         <is>
-          <t>Thay theo tr.40 (BBS cũ 19.981,23 kg, bản vẽ 19.648,73 kg)</t>
+          <t>Thay theo tr.40 (BBS cũ 19.981,23 kg, bản vẽ 19.885,78 kg)</t>
         </is>
       </c>
     </row>
@@ -7161,7 +7161,7 @@
       </c>
       <c r="R94" s="5" t="inlineStr">
         <is>
-          <t>Thay theo tr.40 (BBS cũ 19.981,23 kg, bản vẽ 19.648,73 kg)</t>
+          <t>Thay theo tr.40 (BBS cũ 19.981,23 kg, bản vẽ 19.885,78 kg)</t>
         </is>
       </c>
     </row>
@@ -7237,7 +7237,7 @@
       </c>
       <c r="R95" s="5" t="inlineStr">
         <is>
-          <t>Thay theo tr.40 (BBS cũ 19.981,23 kg, bản vẽ 19.648,73 kg)</t>
+          <t>Thay theo tr.40 (BBS cũ 19.981,23 kg, bản vẽ 19.885,78 kg)</t>
         </is>
       </c>
     </row>
@@ -7313,7 +7313,7 @@
       </c>
       <c r="R96" s="5" t="inlineStr">
         <is>
-          <t>Thay theo tr.40 (BBS cũ 19.981,23 kg, bản vẽ 19.648,73 kg)</t>
+          <t>Thay theo tr.40 (BBS cũ 19.981,23 kg, bản vẽ 19.885,78 kg)</t>
         </is>
       </c>
     </row>
@@ -7389,7 +7389,7 @@
       </c>
       <c r="R97" s="5" t="inlineStr">
         <is>
-          <t>Thay theo tr.40 (BBS cũ 19.981,23 kg, bản vẽ 19.648,73 kg)</t>
+          <t>Thay theo tr.40 (BBS cũ 19.981,23 kg, bản vẽ 19.885,78 kg)</t>
         </is>
       </c>
     </row>
@@ -7465,7 +7465,7 @@
       </c>
       <c r="R98" s="5" t="inlineStr">
         <is>
-          <t>Thay theo tr.40 (BBS cũ 19.981,23 kg, bản vẽ 19.648,73 kg)</t>
+          <t>Thay theo tr.40 (BBS cũ 19.981,23 kg, bản vẽ 19.885,78 kg)</t>
         </is>
       </c>
     </row>
@@ -7541,7 +7541,7 @@
       </c>
       <c r="R99" s="5" t="inlineStr">
         <is>
-          <t>Thay theo tr.40 (BBS cũ 19.981,23 kg, bản vẽ 19.648,73 kg)</t>
+          <t>Thay theo tr.40 (BBS cũ 19.981,23 kg, bản vẽ 19.885,78 kg)</t>
         </is>
       </c>
     </row>
@@ -7617,7 +7617,7 @@
       </c>
       <c r="R100" s="5" t="inlineStr">
         <is>
-          <t>Thay theo tr.40 (BBS cũ 19.981,23 kg, bản vẽ 19.648,73 kg)</t>
+          <t>Thay theo tr.40 (BBS cũ 19.981,23 kg, bản vẽ 19.885,78 kg)</t>
         </is>
       </c>
     </row>
@@ -7693,7 +7693,7 @@
       </c>
       <c r="R101" s="5" t="inlineStr">
         <is>
-          <t>Thay theo tr.40 (BBS cũ 19.981,23 kg, bản vẽ 19.648,73 kg)</t>
+          <t>Thay theo tr.40 (BBS cũ 19.981,23 kg, bản vẽ 19.885,78 kg)</t>
         </is>
       </c>
     </row>
@@ -7769,7 +7769,7 @@
       </c>
       <c r="R102" s="5" t="inlineStr">
         <is>
-          <t>Thay theo tr.40 (BBS cũ 19.981,23 kg, bản vẽ 19.648,73 kg)</t>
+          <t>Thay theo tr.40 (BBS cũ 19.981,23 kg, bản vẽ 19.885,78 kg)</t>
         </is>
       </c>
     </row>
@@ -7845,7 +7845,7 @@
       </c>
       <c r="R103" s="5" t="inlineStr">
         <is>
-          <t>Thay theo tr.40 (BBS cũ 19.981,23 kg, bản vẽ 19.648,73 kg)</t>
+          <t>Thay theo tr.40 (BBS cũ 19.981,23 kg, bản vẽ 19.885,78 kg)</t>
         </is>
       </c>
     </row>
@@ -7921,7 +7921,7 @@
       </c>
       <c r="R104" s="5" t="inlineStr">
         <is>
-          <t>Thay theo tr.40 (BBS cũ 19.981,23 kg, bản vẽ 19.648,73 kg)</t>
+          <t>Thay theo tr.40 (BBS cũ 19.981,23 kg, bản vẽ 19.885,78 kg)</t>
         </is>
       </c>
     </row>
@@ -7997,7 +7997,7 @@
       </c>
       <c r="R105" s="5" t="inlineStr">
         <is>
-          <t>Thay theo tr.40 (BBS cũ 19.981,23 kg, bản vẽ 19.648,73 kg)</t>
+          <t>Thay theo tr.40 (BBS cũ 19.981,23 kg, bản vẽ 19.885,78 kg)</t>
         </is>
       </c>
     </row>
@@ -8073,7 +8073,7 @@
       </c>
       <c r="R106" s="5" t="inlineStr">
         <is>
-          <t>Thay theo tr.40 (BBS cũ 19.981,23 kg, bản vẽ 19.648,73 kg)</t>
+          <t>Thay theo tr.40 (BBS cũ 19.981,23 kg, bản vẽ 19.885,78 kg)</t>
         </is>
       </c>
     </row>
@@ -8149,7 +8149,7 @@
       </c>
       <c r="R107" s="5" t="inlineStr">
         <is>
-          <t>Thay theo tr.40 (BBS cũ 19.981,23 kg, bản vẽ 19.648,73 kg)</t>
+          <t>Thay theo tr.40 (BBS cũ 19.981,23 kg, bản vẽ 19.885,78 kg)</t>
         </is>
       </c>
     </row>
@@ -8225,7 +8225,7 @@
       </c>
       <c r="R108" s="5" t="inlineStr">
         <is>
-          <t>Thay theo tr.40 (BBS cũ 19.981,23 kg, bản vẽ 19.648,73 kg)</t>
+          <t>Thay theo tr.40 (BBS cũ 19.981,23 kg, bản vẽ 19.885,78 kg)</t>
         </is>
       </c>
     </row>
@@ -8297,7 +8297,7 @@
       </c>
       <c r="R109" s="5" t="inlineStr">
         <is>
-          <t>Thay theo tr.40 (BBS cũ 19.981,23 kg, bản vẽ 19.648,73 kg)</t>
+          <t>Thay theo tr.40 (BBS cũ 19.981,23 kg, bản vẽ 19.885,78 kg)</t>
         </is>
       </c>
     </row>
@@ -8369,7 +8369,7 @@
       </c>
       <c r="R110" s="5" t="inlineStr">
         <is>
-          <t>Thay theo tr.40 (BBS cũ 19.981,23 kg, bản vẽ 19.648,73 kg)</t>
+          <t>Thay theo tr.40 (BBS cũ 19.981,23 kg, bản vẽ 19.885,78 kg)</t>
         </is>
       </c>
     </row>
@@ -8441,7 +8441,7 @@
       </c>
       <c r="R111" s="5" t="inlineStr">
         <is>
-          <t>Thay theo tr.40 (BBS cũ 19.981,23 kg, bản vẽ 19.648,73 kg)</t>
+          <t>Thay theo tr.40 (BBS cũ 19.981,23 kg, bản vẽ 19.885,78 kg)</t>
         </is>
       </c>
     </row>
@@ -8517,7 +8517,7 @@
       </c>
       <c r="R112" s="5" t="inlineStr">
         <is>
-          <t>Thay theo tr.40 (BBS cũ 19.981,23 kg, bản vẽ 19.648,73 kg)</t>
+          <t>Thay theo tr.40 (BBS cũ 19.981,23 kg, bản vẽ 19.885,78 kg)</t>
         </is>
       </c>
     </row>
@@ -8593,7 +8593,7 @@
       </c>
       <c r="R113" s="5" t="inlineStr">
         <is>
-          <t>Thay theo tr.40 (BBS cũ 19.981,23 kg, bản vẽ 19.648,73 kg)</t>
+          <t>Thay theo tr.40 (BBS cũ 19.981,23 kg, bản vẽ 19.885,78 kg)</t>
         </is>
       </c>
     </row>
@@ -8665,7 +8665,7 @@
       </c>
       <c r="R114" s="5" t="inlineStr">
         <is>
-          <t>Thay theo tr.40 (BBS cũ 19.981,23 kg, bản vẽ 19.648,73 kg)</t>
+          <t>Thay theo tr.40 (BBS cũ 19.981,23 kg, bản vẽ 19.885,78 kg)</t>
         </is>
       </c>
     </row>
@@ -8737,7 +8737,7 @@
       </c>
       <c r="R115" s="5" t="inlineStr">
         <is>
-          <t>Thay theo tr.40 (BBS cũ 19.981,23 kg, bản vẽ 19.648,73 kg)</t>
+          <t>Thay theo tr.40 (BBS cũ 19.981,23 kg, bản vẽ 19.885,78 kg)</t>
         </is>
       </c>
     </row>
@@ -8813,7 +8813,7 @@
       </c>
       <c r="R116" s="5" t="inlineStr">
         <is>
-          <t>Thay theo tr.40 (BBS cũ 19.981,23 kg, bản vẽ 19.648,73 kg)</t>
+          <t>Thay theo tr.40 (BBS cũ 19.981,23 kg, bản vẽ 19.885,78 kg)</t>
         </is>
       </c>
     </row>
@@ -8889,7 +8889,7 @@
       </c>
       <c r="R117" s="5" t="inlineStr">
         <is>
-          <t>Thay theo tr.40 (BBS cũ 19.981,23 kg, bản vẽ 19.648,73 kg)</t>
+          <t>Thay theo tr.40 (BBS cũ 19.981,23 kg, bản vẽ 19.885,78 kg)</t>
         </is>
       </c>
     </row>
@@ -8965,7 +8965,7 @@
       </c>
       <c r="R118" s="5" t="inlineStr">
         <is>
-          <t>Thay theo tr.40 (BBS cũ 19.981,23 kg, bản vẽ 19.648,73 kg)</t>
+          <t>Thay theo tr.40 (BBS cũ 19.981,23 kg, bản vẽ 19.885,78 kg)</t>
         </is>
       </c>
     </row>
@@ -9037,7 +9037,7 @@
       </c>
       <c r="R119" s="5" t="inlineStr">
         <is>
-          <t>Thay theo tr.40 (BBS cũ 19.981,23 kg, bản vẽ 19.648,73 kg) | BẢN VẼ ghi khối lượng 0 dù dài × SL × kg/m = 51.50 kg — sai trên bản vẽ — xem PDF tr.40 | BBS vẫn giữ thanh này để gia công (có dài và số lượng trên bản vẽ) nên BBS lớn hơn tổng bản vẽ phần này — chủ dự án quyết định và ghim</t>
+          <t>Thay theo tr.40 (BBS cũ 19.981,23 kg, bản vẽ 19.885,78 kg) | BẢN VẼ ghi khối lượng 0 dù dài × SL × kg/m = 51.50 kg — sai trên bản vẽ — xem PDF tr.40 | Chủ dự án quyết định 11/10/2026: tính các thanh này (bản vẽ ghi 0 kg là sai sót)</t>
         </is>
       </c>
     </row>
@@ -9109,7 +9109,7 @@
       </c>
       <c r="R120" s="5" t="inlineStr">
         <is>
-          <t>Thay theo tr.40 (BBS cũ 19.981,23 kg, bản vẽ 19.648,73 kg) | BẢN VẼ ghi khối lượng 0 dù dài × SL × kg/m = 48.84 kg — sai trên bản vẽ — xem PDF tr.40 | BBS vẫn giữ thanh này để gia công (có dài và số lượng trên bản vẽ) nên BBS lớn hơn tổng bản vẽ phần này — chủ dự án quyết định và ghim</t>
+          <t>Thay theo tr.40 (BBS cũ 19.981,23 kg, bản vẽ 19.885,78 kg) | BẢN VẼ ghi khối lượng 0 dù dài × SL × kg/m = 48.84 kg — sai trên bản vẽ — xem PDF tr.40 | Chủ dự án quyết định 11/10/2026: tính các thanh này (bản vẽ ghi 0 kg là sai sót)</t>
         </is>
       </c>
     </row>
@@ -9185,7 +9185,7 @@
       </c>
       <c r="R121" s="5" t="inlineStr">
         <is>
-          <t>Thay theo tr.40 (BBS cũ 19.981,23 kg, bản vẽ 19.648,73 kg)</t>
+          <t>Thay theo tr.40 (BBS cũ 19.981,23 kg, bản vẽ 19.885,78 kg)</t>
         </is>
       </c>
     </row>
@@ -9257,7 +9257,7 @@
       </c>
       <c r="R122" s="5" t="inlineStr">
         <is>
-          <t>Thay theo tr.40 (BBS cũ 19.981,23 kg, bản vẽ 19.648,73 kg) | BẢN VẼ ghi khối lượng 0 dù dài × SL × kg/m = 136.71 kg — sai trên bản vẽ — xem PDF tr.40 | BBS vẫn giữ thanh này để gia công (có dài và số lượng trên bản vẽ) nên BBS lớn hơn tổng bản vẽ phần này — chủ dự án quyết định và ghim</t>
+          <t>Thay theo tr.40 (BBS cũ 19.981,23 kg, bản vẽ 19.885,78 kg) | BẢN VẼ ghi khối lượng 0 dù dài × SL × kg/m = 136.71 kg — sai trên bản vẽ — xem PDF tr.40 | Chủ dự án quyết định 11/10/2026: tính các thanh này (bản vẽ ghi 0 kg là sai sót)</t>
         </is>
       </c>
     </row>
@@ -9333,7 +9333,7 @@
       </c>
       <c r="R123" s="5" t="inlineStr">
         <is>
-          <t>Thay theo tr.40 (BBS cũ 19.981,23 kg, bản vẽ 19.648,73 kg)</t>
+          <t>Thay theo tr.40 (BBS cũ 19.981,23 kg, bản vẽ 19.885,78 kg)</t>
         </is>
       </c>
     </row>
@@ -9409,7 +9409,7 @@
       </c>
       <c r="R124" s="5" t="inlineStr">
         <is>
-          <t>Thay theo tr.40 (BBS cũ 19.981,23 kg, bản vẽ 19.648,73 kg)</t>
+          <t>Thay theo tr.40 (BBS cũ 19.981,23 kg, bản vẽ 19.885,78 kg)</t>
         </is>
       </c>
     </row>
@@ -9485,7 +9485,7 @@
       </c>
       <c r="R125" s="5" t="inlineStr">
         <is>
-          <t>Thay theo tr.40 (BBS cũ 19.981,23 kg, bản vẽ 19.648,73 kg)</t>
+          <t>Thay theo tr.40 (BBS cũ 19.981,23 kg, bản vẽ 19.885,78 kg)</t>
         </is>
       </c>
     </row>
@@ -9557,7 +9557,7 @@
       </c>
       <c r="R126" s="5" t="inlineStr">
         <is>
-          <t>Thay theo tr.40 (BBS cũ 19.981,23 kg, bản vẽ 19.648,73 kg) | OCR tách chiều dài thành '164' và '0' → 1640 mm; số lượng trống/không đọc được, suy = khối lượng ghi ÷ (dài × kg/m) = 4 — Σ bảng sau sửa khớp tổng bản vẽ — xem PDF tr.40</t>
+          <t>Thay theo tr.40 (BBS cũ 19.981,23 kg, bản vẽ 19.885,78 kg) | OCR tách chiều dài thành '164' và '0' → 1640 mm; số lượng trống/không đọc được, suy = khối lượng ghi ÷ (dài × kg/m) = 4 — Σ bảng sau sửa khớp tổng bản vẽ — xem PDF tr.40</t>
         </is>
       </c>
     </row>
@@ -9633,7 +9633,7 @@
       </c>
       <c r="R127" s="5" t="inlineStr">
         <is>
-          <t>Thay theo tr.40 (BBS cũ 19.981,23 kg, bản vẽ 19.648,73 kg) | OCR tách chiều dài thành '64' và '0' → 640 mm; kg/m không đọc được, lấy 0.395 như các thanh Ø8 khác của bảng; khối lượng 1 cấu kiện không đọc được, lấy từ cột tổng (12.64); số lượng trống/không đọc được, suy = khối lượng ghi ÷ (dài × kg/m) = 50 — Σ bảng sau sửa khớp tổng bản vẽ — xem PDF tr.40</t>
+          <t>Thay theo tr.40 (BBS cũ 19.981,23 kg, bản vẽ 19.885,78 kg) | OCR tách chiều dài thành '64' và '0' → 640 mm; kg/m không đọc được, lấy 0.395 như các thanh Ø8 khác của bảng; khối lượng 1 cấu kiện không đọc được, lấy từ cột tổng (12.64); số lượng trống/không đọc được, suy = khối lượng ghi ÷ (dài × kg/m) = 50 — Σ bảng sau sửa khớp tổng bản vẽ — xem PDF tr.40</t>
         </is>
       </c>
     </row>
@@ -9709,7 +9709,7 @@
       </c>
       <c r="R128" s="5" t="inlineStr">
         <is>
-          <t>Thay theo tr.40 (BBS cũ 19.981,23 kg, bản vẽ 19.648,73 kg) | OCR tách chiều dài thành '48' và '0' → 480 mm; khối lượng 1 cấu kiện trống, lấy từ cột tổng (12.32) — Σ bảng sau sửa khớp tổng bản vẽ — xem PDF tr.40</t>
+          <t>Thay theo tr.40 (BBS cũ 19.981,23 kg, bản vẽ 19.885,78 kg) | OCR tách chiều dài thành '48' và '0' → 480 mm; khối lượng 1 cấu kiện trống, lấy từ cột tổng (12.32) — Σ bảng sau sửa khớp tổng bản vẽ — xem PDF tr.40</t>
         </is>
       </c>
     </row>
@@ -9785,7 +9785,7 @@
       </c>
       <c r="R129" s="5" t="inlineStr">
         <is>
-          <t>Thay theo tr.40 (BBS cũ 19.981,23 kg, bản vẽ 19.648,73 kg) | OCR tách chiều dài thành '189' và '0' → 1890 mm; kg/m không đọc được, lấy 1.58 như các thanh Ø16 khác của bảng; khối lượng 1 cấu kiện không đọc được, lấy từ cột tổng (20.90); số lượng trống/không đọc được, suy = khối lượng ghi ÷ (dài × kg/m) = 7 — Σ bảng sau sửa khớp tổng bản vẽ — xem PDF tr.40</t>
+          <t>Thay theo tr.40 (BBS cũ 19.981,23 kg, bản vẽ 19.885,78 kg) | OCR tách chiều dài thành '189' và '0' → 1890 mm; kg/m không đọc được, lấy 1.58 như các thanh Ø16 khác của bảng; khối lượng 1 cấu kiện không đọc được, lấy từ cột tổng (20.90); số lượng trống/không đọc được, suy = khối lượng ghi ÷ (dài × kg/m) = 7 — Σ bảng sau sửa khớp tổng bản vẽ — xem PDF tr.40</t>
         </is>
       </c>
     </row>
@@ -9861,7 +9861,7 @@
       </c>
       <c r="R130" s="5" t="inlineStr">
         <is>
-          <t>Thay theo tr.40 (BBS cũ 19.981,23 kg, bản vẽ 19.648,73 kg) | OCR tách chiều dài thành '159' và '0' → 1590 mm — Σ bảng sau sửa khớp tổng bản vẽ — xem PDF tr.40</t>
+          <t>Thay theo tr.40 (BBS cũ 19.981,23 kg, bản vẽ 19.885,78 kg) | OCR tách chiều dài thành '159' và '0' → 1590 mm — Σ bảng sau sửa khớp tổng bản vẽ — xem PDF tr.40</t>
         </is>
       </c>
     </row>
@@ -31956,13 +31956,13 @@
         <v>0</v>
       </c>
       <c r="F5" s="10" t="n">
-        <v>19648.73</v>
+        <v>19885.78</v>
       </c>
       <c r="G5" s="10" t="n">
         <v>19876.96</v>
       </c>
       <c r="H5" s="10" t="n">
-        <v>228.23</v>
+        <v>-8.82</v>
       </c>
       <c r="I5" s="10" t="inlineStr"/>
     </row>
@@ -32414,7 +32414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I76"/>
+  <dimension ref="A1:I77"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -32570,17 +32570,17 @@
       <c r="D7" t="inlineStr"/>
       <c r="E7" s="11" t="inlineStr">
         <is>
-          <t>THAY THEO BẢN VẼ: BBS cũ 19.981,23 kg; bản vẽ 19.648,73 kg</t>
+          <t>Bản vẽ ghi 0 kg cho một số thanh (dài × SL × kg/m = 237,05 kg); Chủ dự án quyết định 11/10/2026: tính các thanh này (bản vẽ ghi 0 kg là sai sót) → tổng đối chiếu = tổng bản vẽ + 237,05 kg</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>19.981,23 kg</t>
+          <t>19.648,73 kg</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>19.648,73 kg</t>
+          <t>19.885,78 kg</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
@@ -32597,28 +32597,28 @@
       <c r="B8" t="inlineStr"/>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Trụ T1, T2 (Bệ móng)</t>
+          <t>Mố M2</t>
         </is>
       </c>
       <c r="D8" t="inlineStr"/>
       <c r="E8" s="11" t="inlineStr">
         <is>
-          <t>THAY THEO BẢN VẼ: BBS cũ 18.877,75 kg; bản vẽ 32.355,66 kg</t>
+          <t>THAY THEO BẢN VẼ: BBS cũ 19.981,23 kg; bản vẽ 19.885,78 kg</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>18.877,75 kg</t>
+          <t>19.981,23 kg</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>32.355,66 kg</t>
+          <t>19.885,78 kg</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>tr.44, tr.55</t>
+          <t>tr.40</t>
         </is>
       </c>
       <c r="I8" t="inlineStr"/>
@@ -32630,28 +32630,28 @@
       <c r="B9" t="inlineStr"/>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Trụ T1, T2 (Xà mũ trụ)</t>
+          <t>Trụ T1, T2 (Bệ móng)</t>
         </is>
       </c>
       <c r="D9" t="inlineStr"/>
       <c r="E9" s="11" t="inlineStr">
         <is>
-          <t>THAY THEO BẢN VẼ: BBS cũ 88.347,00 kg; bản vẽ 26.026,22 kg</t>
+          <t>THAY THEO BẢN VẼ: BBS cũ 18.877,75 kg; bản vẽ 32.355,66 kg</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>88.347,00 kg</t>
+          <t>18.877,75 kg</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>26.026,22 kg</t>
+          <t>32.355,66 kg</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>tr.51, tr.62</t>
+          <t>tr.44, tr.55</t>
         </is>
       </c>
       <c r="I9" t="inlineStr"/>
@@ -32663,20 +32663,28 @@
       <c r="B10" t="inlineStr"/>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Dầm chủ Super-T (15 phiến L=38.2m)</t>
+          <t>Trụ T1, T2 (Xà mũ trụ)</t>
         </is>
       </c>
       <c r="D10" t="inlineStr"/>
       <c r="E10" s="11" t="inlineStr">
         <is>
-          <t>Số cấu kiện cần xác nhận: Số phiến 3 S1B1 + 3 S1B2 + 9 S1G suy từ bảng tổng hợp toàn cầu tr.175 (dấu thẩm tra): 3×6.071,25 + 3×6.065,28 + 9×5.920,08 = 89.690,31 kg = 77,743 + 11,947 t — xác nhận theo mặt cắt ngang bố trí dầm.</t>
-        </is>
-      </c>
-      <c r="F10" t="inlineStr"/>
-      <c r="G10" t="inlineStr"/>
+          <t>THAY THEO BẢN VẼ: BBS cũ 88.347,00 kg; bản vẽ 26.026,22 kg</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>88.347,00 kg</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>26.026,22 kg</t>
+        </is>
+      </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>tr.88, tr.91, tr.94</t>
+          <t>tr.51, tr.62</t>
         </is>
       </c>
       <c r="I10" t="inlineStr"/>
@@ -32694,19 +32702,11 @@
       <c r="D11" t="inlineStr"/>
       <c r="E11" s="11" t="inlineStr">
         <is>
-          <t>THAY THEO BẢN VẼ: BBS cũ 361.596,10 kg; bản vẽ 89.690,31 kg</t>
-        </is>
-      </c>
-      <c r="F11" t="inlineStr">
-        <is>
-          <t>361.596,10 kg</t>
-        </is>
-      </c>
-      <c r="G11" t="inlineStr">
-        <is>
-          <t>89.690,31 kg</t>
-        </is>
-      </c>
+          <t>Số cấu kiện cần xác nhận: Số phiến 3 S1B1 + 3 S1B2 + 9 S1G suy từ bảng tổng hợp toàn cầu tr.175 (dấu thẩm tra): 3×6.071,25 + 3×6.065,28 + 9×5.920,08 = 89.690,31 kg = 77,743 + 11,947 t — xác nhận theo mặt cắt ngang bố trí dầm.</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr"/>
+      <c r="G11" t="inlineStr"/>
       <c r="H11" t="inlineStr">
         <is>
           <t>tr.88, tr.91, tr.94</t>
@@ -32721,30 +32721,30 @@
       <c r="B12" t="inlineStr"/>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Dầm ngang (Diaphragm)</t>
-        </is>
-      </c>
-      <c r="D12" t="inlineStr">
-        <is>
-          <t>16</t>
-        </is>
-      </c>
+          <t>Dầm chủ Super-T (15 phiến L=38.2m)</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr"/>
       <c r="E12" s="11" t="inlineStr">
         <is>
-          <t>Dòng BBS cũ sai rõ ràng (Ø không phải thép thanh hoặc dài &lt; 50 mm) — đã loại</t>
+          <t>THAY THEO BẢN VẼ: BBS cũ 361.596,10 kg; bản vẽ 89.690,31 kg</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>Ø128 L=0.002 m × 525 × 1, 106.18 kg/m = 111,49 kg</t>
+          <t>361.596,10 kg</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>đã loại</t>
-        </is>
-      </c>
-      <c r="H12" t="inlineStr"/>
+          <t>89.690,31 kg</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>tr.88, tr.91, tr.94</t>
+        </is>
+      </c>
       <c r="I12" t="inlineStr"/>
     </row>
     <row r="13">
@@ -32759,7 +32759,7 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>20</t>
+          <t>16</t>
         </is>
       </c>
       <c r="E13" s="11" t="inlineStr">
@@ -32769,7 +32769,7 @@
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>Ø32 L=0.002 m × 1450 × 1, 114.61 kg/m = 332,37 kg</t>
+          <t>Ø128 L=0.002 m × 525 × 1, 106.18 kg/m = 111,49 kg</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
@@ -32792,7 +32792,7 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>16</t>
+          <t>20</t>
         </is>
       </c>
       <c r="E14" s="11" t="inlineStr">
@@ -32802,7 +32802,7 @@
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>Ø112 L=0.002 m × 1390 × 1, 245.97 kg/m = 683,80 kg</t>
+          <t>Ø32 L=0.002 m × 1450 × 1, 114.61 kg/m = 332,37 kg</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
@@ -32835,7 +32835,7 @@
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>Ø32 L=0.002 m × 1140 × 1, 57.64 kg/m = 131,42 kg</t>
+          <t>Ø112 L=0.002 m × 1390 × 1, 245.97 kg/m = 683,80 kg</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
@@ -32868,7 +32868,7 @@
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>Ø64 L=0.002 m × 3262 × 1, 329.85 kg/m = 2.151,94 kg</t>
+          <t>Ø32 L=0.002 m × 1140 × 1, 57.64 kg/m = 131,42 kg</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
@@ -32901,7 +32901,7 @@
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>Ø16 L=0.002 m × 2642 × 1, 66.79 kg/m = 352,92 kg</t>
+          <t>Ø64 L=0.002 m × 3262 × 1, 329.85 kg/m = 2.151,94 kg</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
@@ -32922,27 +32922,27 @@
           <t>Dầm ngang (Diaphragm)</t>
         </is>
       </c>
-      <c r="D18" t="inlineStr"/>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>16</t>
+        </is>
+      </c>
       <c r="E18" s="11" t="inlineStr">
         <is>
-          <t>THAY THEO BẢN VẼ: BBS cũ 0,00 kg (+ 6 dòng lỗi 3.763,93 kg); bản vẽ 2.763,12 kg</t>
+          <t>Dòng BBS cũ sai rõ ràng (Ø không phải thép thanh hoặc dài &lt; 50 mm) — đã loại</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>3.763,93 kg</t>
+          <t>Ø16 L=0.002 m × 2642 × 1, 66.79 kg/m = 352,92 kg</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>2.763,12 kg</t>
-        </is>
-      </c>
-      <c r="H18" t="inlineStr">
-        <is>
-          <t>tr.96</t>
-        </is>
-      </c>
+          <t>đã loại</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr"/>
       <c r="I18" t="inlineStr"/>
     </row>
     <row r="19">
@@ -32952,30 +32952,30 @@
       <c r="B19" t="inlineStr"/>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Bản liên tục nhiệt (Link Slab)</t>
-        </is>
-      </c>
-      <c r="D19" t="inlineStr">
-        <is>
-          <t>18</t>
-        </is>
-      </c>
+          <t>Dầm ngang (Diaphragm)</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr"/>
       <c r="E19" s="11" t="inlineStr">
         <is>
-          <t>Dòng BBS cũ sai rõ ràng (Ø không phải thép thanh hoặc dài &lt; 50 mm) — đã loại</t>
+          <t>THAY THEO BẢN VẼ: BBS cũ 0,00 kg (+ 6 dòng lỗi 3.763,93 kg); bản vẽ 2.763,12 kg</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>Ø54 L=0.002 m × 13135 × 1, 1418.58 kg/m = 37.266,10 kg</t>
+          <t>3.763,93 kg</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>đã loại</t>
-        </is>
-      </c>
-      <c r="H19" t="inlineStr"/>
+          <t>2.763,12 kg</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>tr.96</t>
+        </is>
+      </c>
       <c r="I19" t="inlineStr"/>
     </row>
     <row r="20">
@@ -32990,7 +32990,7 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>25</t>
+          <t>18</t>
         </is>
       </c>
       <c r="E20" s="11" t="inlineStr">
@@ -33000,7 +33000,7 @@
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>Ø168 L=0.004 m × 3920 × 1, 2535.46 kg/m = 39.756,01 kg</t>
+          <t>Ø54 L=0.002 m × 13135 × 1, 1418.58 kg/m = 37.266,10 kg</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
@@ -33023,7 +33023,7 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>25</t>
         </is>
       </c>
       <c r="E21" s="11" t="inlineStr">
@@ -33033,7 +33033,7 @@
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>Ø260 L=0.001 m × 320 × 1, 51.33 kg/m = 16,43 kg</t>
+          <t>Ø168 L=0.004 m × 3920 × 1, 2535.46 kg/m = 39.756,01 kg</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
@@ -33056,7 +33056,7 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>18</t>
+          <t>10</t>
         </is>
       </c>
       <c r="E22" s="11" t="inlineStr">
@@ -33066,7 +33066,7 @@
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>Ø108 L=0.002 m × 2100 × 1, 453.6 kg/m = 1.905,12 kg</t>
+          <t>Ø260 L=0.001 m × 320 × 1, 51.33 kg/m = 16,43 kg</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
@@ -33087,27 +33087,27 @@
           <t>Bản liên tục nhiệt (Link Slab)</t>
         </is>
       </c>
-      <c r="D23" t="inlineStr"/>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>18</t>
+        </is>
+      </c>
       <c r="E23" s="11" t="inlineStr">
         <is>
-          <t>THAY THEO BẢN VẼ: BBS cũ 0,00 kg (+ 4 dòng lỗi 78.943,65 kg); bản vẽ 8.917,94 kg</t>
+          <t>Dòng BBS cũ sai rõ ràng (Ø không phải thép thanh hoặc dài &lt; 50 mm) — đã loại</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>78.943,65 kg</t>
+          <t>Ø108 L=0.002 m × 2100 × 1, 453.6 kg/m = 1.905,12 kg</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>8.917,94 kg</t>
-        </is>
-      </c>
-      <c r="H23" t="inlineStr">
-        <is>
-          <t>tr.112</t>
-        </is>
-      </c>
+          <t>đã loại</t>
+        </is>
+      </c>
+      <c r="H23" t="inlineStr"/>
       <c r="I23" t="inlineStr"/>
     </row>
     <row r="24">
@@ -33117,28 +33117,28 @@
       <c r="B24" t="inlineStr"/>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Gờ lan can BTCT</t>
+          <t>Bản liên tục nhiệt (Link Slab)</t>
         </is>
       </c>
       <c r="D24" t="inlineStr"/>
       <c r="E24" s="11" t="inlineStr">
         <is>
-          <t>THAY THEO BẢN VẼ: BBS cũ 1.719,70 kg; bản vẽ 20.069,02 kg</t>
+          <t>THAY THEO BẢN VẼ: BBS cũ 0,00 kg (+ 4 dòng lỗi 78.943,65 kg); bản vẽ 8.917,94 kg</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>1.719,70 kg</t>
+          <t>78.943,65 kg</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>20.069,02 kg</t>
+          <t>8.917,94 kg</t>
         </is>
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>tr.119</t>
+          <t>tr.112</t>
         </is>
       </c>
       <c r="I24" t="inlineStr"/>
@@ -33150,28 +33150,28 @@
       <c r="B25" t="inlineStr"/>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Khe co giãn</t>
+          <t>Gờ lan can BTCT</t>
         </is>
       </c>
       <c r="D25" t="inlineStr"/>
       <c r="E25" s="11" t="inlineStr">
         <is>
-          <t>THAY THEO BẢN VẼ: BBS cũ 0,00 kg; bản vẽ 1.359,80 kg</t>
+          <t>THAY THEO BẢN VẼ: BBS cũ 1.719,70 kg; bản vẽ 20.069,02 kg</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>0,00 kg</t>
+          <t>1.719,70 kg</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>1.359,80 kg</t>
+          <t>20.069,02 kg</t>
         </is>
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>tr.121</t>
+          <t>tr.119</t>
         </is>
       </c>
       <c r="I25" t="inlineStr"/>
@@ -33183,28 +33183,28 @@
       <c r="B26" t="inlineStr"/>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Cọc khoan nhồi D1200 (26 cọc L=872m)</t>
+          <t>Khe co giãn</t>
         </is>
       </c>
       <c r="D26" t="inlineStr"/>
       <c r="E26" s="11" t="inlineStr">
         <is>
-          <t>Tổng các trang chi tiết 108.461,59 kg ≠ bảng tổng hợp tr.175 108.884,00 kg (lệch 422,41 kg). Tr.175: D&lt;=10 10,451 t và D&gt;18 97,451 t khớp đúng 3/7/8/8 cọc; nhóm 10&lt;D&lt;=18 ghi 0,982 t nhưng các trang cọc chỉ có 0,559 t — xem PDF tr.175.</t>
+          <t>THAY THEO BẢN VẼ: BBS cũ 0,00 kg; bản vẽ 1.359,80 kg</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>108.461,59 kg</t>
+          <t>0,00 kg</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>108.884,00 kg</t>
+          <t>1.359,80 kg</t>
         </is>
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>tr.175</t>
+          <t>tr.121</t>
         </is>
       </c>
       <c r="I26" t="inlineStr"/>
@@ -33222,14 +33222,22 @@
       <c r="D27" t="inlineStr"/>
       <c r="E27" s="11" t="inlineStr">
         <is>
-          <t>Số cấu kiện cần xác nhận: Số cọc 3/7/8/8 khớp bảng tổng hợp tr.175 (thép D&lt;=10, D&gt;18 và vữa lấp lòng 14,43 m³ = 3×0,34 + 7×0,59 + 8×0,66 + 8×0,50).</t>
-        </is>
-      </c>
-      <c r="F27" t="inlineStr"/>
-      <c r="G27" t="inlineStr"/>
+          <t>Tổng các trang chi tiết 108.461,59 kg ≠ bảng tổng hợp tr.175 108.884,00 kg (lệch 422,41 kg). Tr.175: D&lt;=10 10,451 t và D&gt;18 97,451 t khớp đúng 3/7/8/8 cọc; nhóm 10&lt;D&lt;=18 ghi 0,982 t nhưng các trang cọc chỉ có 0,559 t — xem PDF tr.175.</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>108.461,59 kg</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>108.884,00 kg</t>
+        </is>
+      </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>tr.64, tr.66, tr.68, tr.70</t>
+          <t>tr.175</t>
         </is>
       </c>
       <c r="I27" t="inlineStr"/>
@@ -33247,19 +33255,11 @@
       <c r="D28" t="inlineStr"/>
       <c r="E28" s="11" t="inlineStr">
         <is>
-          <t>THAY THEO BẢN VẼ: BBS cũ 108.765,99 kg; bản vẽ 108.461,59 kg</t>
-        </is>
-      </c>
-      <c r="F28" t="inlineStr">
-        <is>
-          <t>108.765,99 kg</t>
-        </is>
-      </c>
-      <c r="G28" t="inlineStr">
-        <is>
-          <t>108.461,59 kg</t>
-        </is>
-      </c>
+          <t>Số cấu kiện cần xác nhận: Số cọc 3/7/8/8 khớp bảng tổng hợp tr.175 (thép D&lt;=10, D&gt;18 và vữa lấp lòng 14,43 m³ = 3×0,34 + 7×0,59 + 8×0,66 + 8×0,50).</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr"/>
+      <c r="G28" t="inlineStr"/>
       <c r="H28" t="inlineStr">
         <is>
           <t>tr.64, tr.66, tr.68, tr.70</t>
@@ -33271,27 +33271,33 @@
       <c r="A29" t="n">
         <v>26</v>
       </c>
-      <c r="B29" t="n">
-        <v>44</v>
-      </c>
+      <c r="B29" t="inlineStr"/>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Mố M1</t>
-        </is>
-      </c>
-      <c r="D29" t="inlineStr">
-        <is>
-          <t>B1</t>
-        </is>
-      </c>
+          <t>Cọc khoan nhồi D1200 (26 cọc L=872m)</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr"/>
       <c r="E29" s="11" t="inlineStr">
         <is>
-          <t>OCR ghi Ø 'DB', Ø8 suy từ kg/m 0.395 — Σ bảng sau sửa khớp tổng bản vẽ — xem PDF tr.31</t>
-        </is>
-      </c>
-      <c r="F29" t="inlineStr"/>
-      <c r="G29" t="inlineStr"/>
-      <c r="H29" t="inlineStr"/>
+          <t>THAY THEO BẢN VẼ: BBS cũ 108.765,99 kg; bản vẽ 108.461,59 kg</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>108.765,99 kg</t>
+        </is>
+      </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>108.461,59 kg</t>
+        </is>
+      </c>
+      <c r="H29" t="inlineStr">
+        <is>
+          <t>tr.64, tr.66, tr.68, tr.70</t>
+        </is>
+      </c>
       <c r="I29" t="inlineStr"/>
     </row>
     <row r="30">
@@ -33299,21 +33305,21 @@
         <v>27</v>
       </c>
       <c r="B30" t="n">
-        <v>119</v>
+        <v>44</v>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Mố M2</t>
+          <t>Mố M1</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>W6(T)</t>
+          <t>B1</t>
         </is>
       </c>
       <c r="E30" s="11" t="inlineStr">
         <is>
-          <t>BẢN VẼ ghi khối lượng 0 dù dài × SL × kg/m = 51.50 kg — sai trên bản vẽ — xem PDF tr.40</t>
+          <t>OCR ghi Ø 'DB', Ø8 suy từ kg/m 0.395 — Σ bảng sau sửa khớp tổng bản vẽ — xem PDF tr.31</t>
         </is>
       </c>
       <c r="F30" t="inlineStr"/>
@@ -33340,7 +33346,7 @@
       </c>
       <c r="E31" s="11" t="inlineStr">
         <is>
-          <t>BBS vẫn giữ thanh này để gia công (có dài và số lượng trên bản vẽ) nên BBS lớn hơn tổng bản vẽ phần này — chủ dự án quyết định và ghim</t>
+          <t>BẢN VẼ ghi khối lượng 0 dù dài × SL × kg/m = 51.50 kg — sai trên bản vẽ — xem PDF tr.40</t>
         </is>
       </c>
       <c r="F31" t="inlineStr"/>
@@ -33353,7 +33359,7 @@
         <v>29</v>
       </c>
       <c r="B32" t="n">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="C32" t="inlineStr">
         <is>
@@ -33362,12 +33368,12 @@
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>W7(T)</t>
+          <t>W6(T)</t>
         </is>
       </c>
       <c r="E32" s="11" t="inlineStr">
         <is>
-          <t>BẢN VẼ ghi khối lượng 0 dù dài × SL × kg/m = 48.84 kg — sai trên bản vẽ — xem PDF tr.40</t>
+          <t>Chủ dự án quyết định 11/10/2026: tính các thanh này (bản vẽ ghi 0 kg là sai sót)</t>
         </is>
       </c>
       <c r="F32" t="inlineStr"/>
@@ -33394,7 +33400,7 @@
       </c>
       <c r="E33" s="11" t="inlineStr">
         <is>
-          <t>BBS vẫn giữ thanh này để gia công (có dài và số lượng trên bản vẽ) nên BBS lớn hơn tổng bản vẽ phần này — chủ dự án quyết định và ghim</t>
+          <t>BẢN VẼ ghi khối lượng 0 dù dài × SL × kg/m = 48.84 kg — sai trên bản vẽ — xem PDF tr.40</t>
         </is>
       </c>
       <c r="F33" t="inlineStr"/>
@@ -33407,7 +33413,7 @@
         <v>31</v>
       </c>
       <c r="B34" t="n">
-        <v>122</v>
+        <v>120</v>
       </c>
       <c r="C34" t="inlineStr">
         <is>
@@ -33416,12 +33422,12 @@
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>W9(T)</t>
+          <t>W7(T)</t>
         </is>
       </c>
       <c r="E34" s="11" t="inlineStr">
         <is>
-          <t>BẢN VẼ ghi khối lượng 0 dù dài × SL × kg/m = 136.71 kg — sai trên bản vẽ — xem PDF tr.40</t>
+          <t>Chủ dự án quyết định 11/10/2026: tính các thanh này (bản vẽ ghi 0 kg là sai sót)</t>
         </is>
       </c>
       <c r="F34" t="inlineStr"/>
@@ -33448,7 +33454,7 @@
       </c>
       <c r="E35" s="11" t="inlineStr">
         <is>
-          <t>BBS vẫn giữ thanh này để gia công (có dài và số lượng trên bản vẽ) nên BBS lớn hơn tổng bản vẽ phần này — chủ dự án quyết định và ghim</t>
+          <t>BẢN VẼ ghi khối lượng 0 dù dài × SL × kg/m = 136.71 kg — sai trên bản vẽ — xem PDF tr.40</t>
         </is>
       </c>
       <c r="F35" t="inlineStr"/>
@@ -33461,7 +33467,7 @@
         <v>33</v>
       </c>
       <c r="B36" t="n">
-        <v>126</v>
+        <v>122</v>
       </c>
       <c r="C36" t="inlineStr">
         <is>
@@ -33470,12 +33476,12 @@
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>n</t>
+          <t>W9(T)</t>
         </is>
       </c>
       <c r="E36" s="11" t="inlineStr">
         <is>
-          <t>OCR tách chiều dài thành '164' và '0' → 1640 mm; số lượng trống/không đọc được, suy = khối lượng ghi ÷ (dài × kg/m) = 4 — Σ bảng sau sửa khớp tổng bản vẽ — xem PDF tr.40</t>
+          <t>Chủ dự án quyết định 11/10/2026: tính các thanh này (bản vẽ ghi 0 kg là sai sót)</t>
         </is>
       </c>
       <c r="F36" t="inlineStr"/>
@@ -33488,7 +33494,7 @@
         <v>34</v>
       </c>
       <c r="B37" t="n">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="C37" t="inlineStr">
         <is>
@@ -33497,12 +33503,12 @@
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>B1</t>
+          <t>n</t>
         </is>
       </c>
       <c r="E37" s="11" t="inlineStr">
         <is>
-          <t>OCR tách chiều dài thành '64' và '0' → 640 mm; kg/m không đọc được, lấy 0.395 như các thanh Ø8 khác của bảng; khối lượng 1 cấu kiện không đọc được, lấy từ cột tổng (12.64); số lượng trống/không đọc được, suy = khối lượng ghi ÷ (dài × kg/m) = 50 — Σ bảng sau sửa khớp tổng bản vẽ — xem PDF tr.40</t>
+          <t>OCR tách chiều dài thành '164' và '0' → 1640 mm; số lượng trống/không đọc được, suy = khối lượng ghi ÷ (dài × kg/m) = 4 — Σ bảng sau sửa khớp tổng bản vẽ — xem PDF tr.40</t>
         </is>
       </c>
       <c r="F37" t="inlineStr"/>
@@ -33515,7 +33521,7 @@
         <v>35</v>
       </c>
       <c r="B38" t="n">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="C38" t="inlineStr">
         <is>
@@ -33524,12 +33530,12 @@
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>B2</t>
+          <t>B1</t>
         </is>
       </c>
       <c r="E38" s="11" t="inlineStr">
         <is>
-          <t>OCR tách chiều dài thành '48' và '0' → 480 mm; khối lượng 1 cấu kiện trống, lấy từ cột tổng (12.32) — Σ bảng sau sửa khớp tổng bản vẽ — xem PDF tr.40</t>
+          <t>OCR tách chiều dài thành '64' và '0' → 640 mm; kg/m không đọc được, lấy 0.395 như các thanh Ø8 khác của bảng; khối lượng 1 cấu kiện không đọc được, lấy từ cột tổng (12.64); số lượng trống/không đọc được, suy = khối lượng ghi ÷ (dài × kg/m) = 50 — Σ bảng sau sửa khớp tổng bản vẽ — xem PDF tr.40</t>
         </is>
       </c>
       <c r="F38" t="inlineStr"/>
@@ -33542,7 +33548,7 @@
         <v>36</v>
       </c>
       <c r="B39" t="n">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="C39" t="inlineStr">
         <is>
@@ -33551,12 +33557,12 @@
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>T1</t>
+          <t>B2</t>
         </is>
       </c>
       <c r="E39" s="11" t="inlineStr">
         <is>
-          <t>OCR tách chiều dài thành '189' và '0' → 1890 mm; kg/m không đọc được, lấy 1.58 như các thanh Ø16 khác của bảng; khối lượng 1 cấu kiện không đọc được, lấy từ cột tổng (20.90); số lượng trống/không đọc được, suy = khối lượng ghi ÷ (dài × kg/m) = 7 — Σ bảng sau sửa khớp tổng bản vẽ — xem PDF tr.40</t>
+          <t>OCR tách chiều dài thành '48' và '0' → 480 mm; khối lượng 1 cấu kiện trống, lấy từ cột tổng (12.32) — Σ bảng sau sửa khớp tổng bản vẽ — xem PDF tr.40</t>
         </is>
       </c>
       <c r="F39" t="inlineStr"/>
@@ -33569,7 +33575,7 @@
         <v>37</v>
       </c>
       <c r="B40" t="n">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="C40" t="inlineStr">
         <is>
@@ -33578,12 +33584,12 @@
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>T2</t>
+          <t>T1</t>
         </is>
       </c>
       <c r="E40" s="11" t="inlineStr">
         <is>
-          <t>OCR tách chiều dài thành '159' và '0' → 1590 mm — Σ bảng sau sửa khớp tổng bản vẽ — xem PDF tr.40</t>
+          <t>OCR tách chiều dài thành '189' và '0' → 1890 mm; kg/m không đọc được, lấy 1.58 như các thanh Ø16 khác của bảng; khối lượng 1 cấu kiện không đọc được, lấy từ cột tổng (20.90); số lượng trống/không đọc được, suy = khối lượng ghi ÷ (dài × kg/m) = 7 — Σ bảng sau sửa khớp tổng bản vẽ — xem PDF tr.40</t>
         </is>
       </c>
       <c r="F40" t="inlineStr"/>
@@ -33596,21 +33602,21 @@
         <v>38</v>
       </c>
       <c r="B41" t="n">
-        <v>134</v>
+        <v>130</v>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>Trụ T1, T2 (Bệ móng)</t>
+          <t>Mố M2</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>(?)</t>
+          <t>T2</t>
         </is>
       </c>
       <c r="E41" s="11" t="inlineStr">
         <is>
-          <t>OCR không đọc được ký hiệu thanh (STT 4) — xem PDF tr.44</t>
+          <t>OCR tách chiều dài thành '159' và '0' → 1590 mm — Σ bảng sau sửa khớp tổng bản vẽ — xem PDF tr.40</t>
         </is>
       </c>
       <c r="F41" t="inlineStr"/>
@@ -33623,11 +33629,11 @@
         <v>39</v>
       </c>
       <c r="B42" t="n">
-        <v>181</v>
+        <v>134</v>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>Trụ T1, T2 (Xà mũ trụ)</t>
+          <t>Trụ T1, T2 (Bệ móng)</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
@@ -33637,7 +33643,7 @@
       </c>
       <c r="E42" s="11" t="inlineStr">
         <is>
-          <t>OCR không đọc được ký hiệu thanh (STT 5) — xem PDF tr.51</t>
+          <t>OCR không đọc được ký hiệu thanh (STT 4) — xem PDF tr.44</t>
         </is>
       </c>
       <c r="F42" t="inlineStr"/>
@@ -33650,7 +33656,7 @@
         <v>40</v>
       </c>
       <c r="B43" t="n">
-        <v>202</v>
+        <v>181</v>
       </c>
       <c r="C43" t="inlineStr">
         <is>
@@ -33664,7 +33670,7 @@
       </c>
       <c r="E43" s="11" t="inlineStr">
         <is>
-          <t>OCR không đọc được ký hiệu thanh (STT 5) — xem PDF tr.62</t>
+          <t>OCR không đọc được ký hiệu thanh (STT 5) — xem PDF tr.51</t>
         </is>
       </c>
       <c r="F43" t="inlineStr"/>
@@ -33677,21 +33683,21 @@
         <v>41</v>
       </c>
       <c r="B44" t="n">
-        <v>233</v>
+        <v>202</v>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>Dầm chủ Super-T (15 phiến L=38.2m)</t>
+          <t>Trụ T1, T2 (Xà mũ trụ)</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>G6a</t>
+          <t>(?)</t>
         </is>
       </c>
       <c r="E44" s="11" t="inlineStr">
         <is>
-          <t>OCR đọc SL = 6, phép tính bản vẽ cho 9 (khối lượng ghi ÷ dài ÷ kg/m) — Σ bảng sau sửa khớp tổng bản vẽ — xem PDF tr.88</t>
+          <t>OCR không đọc được ký hiệu thanh (STT 5) — xem PDF tr.62</t>
         </is>
       </c>
       <c r="F44" t="inlineStr"/>
@@ -33704,7 +33710,7 @@
         <v>42</v>
       </c>
       <c r="B45" t="n">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="C45" t="inlineStr">
         <is>
@@ -33713,12 +33719,12 @@
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>G6b</t>
+          <t>G6a</t>
         </is>
       </c>
       <c r="E45" s="11" t="inlineStr">
         <is>
-          <t>số lượng trống/không đọc được, suy = khối lượng ghi ÷ (dài × kg/m) = 3 — Σ bảng sau sửa khớp tổng bản vẽ — xem PDF tr.88</t>
+          <t>OCR đọc SL = 6, phép tính bản vẽ cho 9 (khối lượng ghi ÷ dài ÷ kg/m) — Σ bảng sau sửa khớp tổng bản vẽ — xem PDF tr.88</t>
         </is>
       </c>
       <c r="F45" t="inlineStr"/>
@@ -33731,7 +33737,7 @@
         <v>43</v>
       </c>
       <c r="B46" t="n">
-        <v>263</v>
+        <v>234</v>
       </c>
       <c r="C46" t="inlineStr">
         <is>
@@ -33740,12 +33746,12 @@
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>Thanh neo</t>
+          <t>G6b</t>
         </is>
       </c>
       <c r="E46" s="11" t="inlineStr">
         <is>
-          <t>OCR đọc khối lượng = 217, dài × SL × kg/m = 2.17 — Σ bảng sau sửa khớp tổng bản vẽ — xem PDF tr.91</t>
+          <t>số lượng trống/không đọc được, suy = khối lượng ghi ÷ (dài × kg/m) = 3 — Σ bảng sau sửa khớp tổng bản vẽ — xem PDF tr.88</t>
         </is>
       </c>
       <c r="F46" t="inlineStr"/>
@@ -33758,7 +33764,7 @@
         <v>44</v>
       </c>
       <c r="B47" t="n">
-        <v>277</v>
+        <v>263</v>
       </c>
       <c r="C47" t="inlineStr">
         <is>
@@ -33767,12 +33773,12 @@
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>(?)</t>
+          <t>Thanh neo</t>
         </is>
       </c>
       <c r="E47" s="11" t="inlineStr">
         <is>
-          <t>OCR không đọc được ký hiệu thanh (STT ?) — xem PDF tr.94</t>
+          <t>OCR đọc khối lượng = 217, dài × SL × kg/m = 2.17 — Σ bảng sau sửa khớp tổng bản vẽ — xem PDF tr.91</t>
         </is>
       </c>
       <c r="F47" t="inlineStr"/>
@@ -33785,7 +33791,7 @@
         <v>45</v>
       </c>
       <c r="B48" t="n">
-        <v>279</v>
+        <v>277</v>
       </c>
       <c r="C48" t="inlineStr">
         <is>
@@ -33794,12 +33800,12 @@
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>G6b</t>
+          <t>(?)</t>
         </is>
       </c>
       <c r="E48" s="11" t="inlineStr">
         <is>
-          <t>số lượng trống/không đọc được, suy = khối lượng ghi ÷ (dài × kg/m) = 3 — Σ bảng sau sửa khớp tổng bản vẽ — xem PDF tr.94</t>
+          <t>OCR không đọc được ký hiệu thanh (STT ?) — xem PDF tr.94</t>
         </is>
       </c>
       <c r="F48" t="inlineStr"/>
@@ -33812,21 +33818,21 @@
         <v>46</v>
       </c>
       <c r="B49" t="n">
-        <v>289</v>
+        <v>279</v>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>Dầm ngang (Diaphragm)</t>
+          <t>Dầm chủ Super-T (15 phiến L=38.2m)</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>A1</t>
+          <t>G6b</t>
         </is>
       </c>
       <c r="E49" s="11" t="inlineStr">
         <is>
-          <t>hệ số 3 suy từ cột tổng (318.54 ÷ 106.18) — xem PDF tr.96</t>
+          <t>số lượng trống/không đọc được, suy = khối lượng ghi ÷ (dài × kg/m) = 3 — Σ bảng sau sửa khớp tổng bản vẽ — xem PDF tr.94</t>
         </is>
       </c>
       <c r="F49" t="inlineStr"/>
@@ -33839,7 +33845,7 @@
         <v>47</v>
       </c>
       <c r="B50" t="n">
-        <v>290</v>
+        <v>289</v>
       </c>
       <c r="C50" t="inlineStr">
         <is>
@@ -33848,12 +33854,12 @@
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>A2</t>
+          <t>A1</t>
         </is>
       </c>
       <c r="E50" s="11" t="inlineStr">
         <is>
-          <t>hệ số 3 suy từ cột tổng (343.83 ÷ 114.61) — xem PDF tr.96</t>
+          <t>hệ số 3 suy từ cột tổng (318.54 ÷ 106.18) — xem PDF tr.96</t>
         </is>
       </c>
       <c r="F50" t="inlineStr"/>
@@ -33866,7 +33872,7 @@
         <v>48</v>
       </c>
       <c r="B51" t="n">
-        <v>291</v>
+        <v>290</v>
       </c>
       <c r="C51" t="inlineStr">
         <is>
@@ -33875,12 +33881,12 @@
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>A3</t>
+          <t>A2</t>
         </is>
       </c>
       <c r="E51" s="11" t="inlineStr">
         <is>
-          <t>hệ số 3 suy từ cột tổng (737.91 ÷ 245.97) — xem PDF tr.96</t>
+          <t>hệ số 3 suy từ cột tổng (343.83 ÷ 114.61) — xem PDF tr.96</t>
         </is>
       </c>
       <c r="F51" t="inlineStr"/>
@@ -33893,7 +33899,7 @@
         <v>49</v>
       </c>
       <c r="B52" t="n">
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="C52" t="inlineStr">
         <is>
@@ -33902,12 +33908,12 @@
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>A4</t>
+          <t>A3</t>
         </is>
       </c>
       <c r="E52" s="11" t="inlineStr">
         <is>
-          <t>hệ số 3 suy từ cột tổng (172.92 ÷ 57.64) — xem PDF tr.96</t>
+          <t>hệ số 3 suy từ cột tổng (737.91 ÷ 245.97) — xem PDF tr.96</t>
         </is>
       </c>
       <c r="F52" t="inlineStr"/>
@@ -33920,7 +33926,7 @@
         <v>50</v>
       </c>
       <c r="B53" t="n">
-        <v>293</v>
+        <v>292</v>
       </c>
       <c r="C53" t="inlineStr">
         <is>
@@ -33929,12 +33935,12 @@
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>A5</t>
+          <t>A4</t>
         </is>
       </c>
       <c r="E53" s="11" t="inlineStr">
         <is>
-          <t>hệ số 3 suy từ cột tổng (989.55 ÷ 329.85) — xem PDF tr.96</t>
+          <t>hệ số 3 suy từ cột tổng (172.92 ÷ 57.64) — xem PDF tr.96</t>
         </is>
       </c>
       <c r="F53" t="inlineStr"/>
@@ -33947,7 +33953,7 @@
         <v>51</v>
       </c>
       <c r="B54" t="n">
-        <v>294</v>
+        <v>293</v>
       </c>
       <c r="C54" t="inlineStr">
         <is>
@@ -33956,12 +33962,12 @@
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>A6</t>
+          <t>A5</t>
         </is>
       </c>
       <c r="E54" s="11" t="inlineStr">
         <is>
-          <t>hệ số 3 suy từ cột tổng (200.37 ÷ 66.79) — xem PDF tr.96</t>
+          <t>hệ số 3 suy từ cột tổng (989.55 ÷ 329.85) — xem PDF tr.96</t>
         </is>
       </c>
       <c r="F54" t="inlineStr"/>
@@ -33974,21 +33980,21 @@
         <v>52</v>
       </c>
       <c r="B55" t="n">
-        <v>318</v>
+        <v>294</v>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>Bản liên tục nhiệt (Link Slab)</t>
+          <t>Dầm ngang (Diaphragm)</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>L1</t>
+          <t>A6</t>
         </is>
       </c>
       <c r="E55" s="11" t="inlineStr">
         <is>
-          <t>hệ số 2 suy từ cột tổng (2,837.16 ÷ 1,418.58) — xem PDF tr.112</t>
+          <t>hệ số 3 suy từ cột tổng (200.37 ÷ 66.79) — xem PDF tr.96</t>
         </is>
       </c>
       <c r="F55" t="inlineStr"/>
@@ -34015,7 +34021,7 @@
       </c>
       <c r="E56" s="11" t="inlineStr">
         <is>
-          <t>OCR ghi Ø 'D1', Ø18 suy từ kg/m 2 — Σ bảng sau sửa khớp tổng bản vẽ — xem PDF tr.112</t>
+          <t>hệ số 2 suy từ cột tổng (2,837.16 ÷ 1,418.58) — xem PDF tr.112</t>
         </is>
       </c>
       <c r="F56" t="inlineStr"/>
@@ -34028,7 +34034,7 @@
         <v>54</v>
       </c>
       <c r="B57" t="n">
-        <v>319</v>
+        <v>318</v>
       </c>
       <c r="C57" t="inlineStr">
         <is>
@@ -34037,12 +34043,12 @@
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>L2</t>
+          <t>L1</t>
         </is>
       </c>
       <c r="E57" s="11" t="inlineStr">
         <is>
-          <t>hệ số 2 suy từ cột tổng (5,070.92 ÷ 2,535.46) — xem PDF tr.112</t>
+          <t>OCR ghi Ø 'D1', Ø18 suy từ kg/m 2 — Σ bảng sau sửa khớp tổng bản vẽ — xem PDF tr.112</t>
         </is>
       </c>
       <c r="F57" t="inlineStr"/>
@@ -34055,7 +34061,7 @@
         <v>55</v>
       </c>
       <c r="B58" t="n">
-        <v>320</v>
+        <v>319</v>
       </c>
       <c r="C58" t="inlineStr">
         <is>
@@ -34064,12 +34070,12 @@
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>L3</t>
+          <t>L2</t>
         </is>
       </c>
       <c r="E58" s="11" t="inlineStr">
         <is>
-          <t>hệ số 2 suy từ cột tổng (102.66 ÷ 51.33) — xem PDF tr.112</t>
+          <t>hệ số 2 suy từ cột tổng (5,070.92 ÷ 2,535.46) — xem PDF tr.112</t>
         </is>
       </c>
       <c r="F58" t="inlineStr"/>
@@ -34082,7 +34088,7 @@
         <v>56</v>
       </c>
       <c r="B59" t="n">
-        <v>321</v>
+        <v>320</v>
       </c>
       <c r="C59" t="inlineStr">
         <is>
@@ -34091,12 +34097,12 @@
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>S4</t>
+          <t>L3</t>
         </is>
       </c>
       <c r="E59" s="11" t="inlineStr">
         <is>
-          <t>hệ số 2 suy từ cột tổng (907.20 ÷ 453.60) — xem PDF tr.112</t>
+          <t>hệ số 2 suy từ cột tổng (102.66 ÷ 51.33) — xem PDF tr.112</t>
         </is>
       </c>
       <c r="F59" t="inlineStr"/>
@@ -34109,21 +34115,21 @@
         <v>57</v>
       </c>
       <c r="B60" t="n">
-        <v>337</v>
+        <v>321</v>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>Gờ lan can BTCT</t>
+          <t>Bản liên tục nhiệt (Link Slab)</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>G1</t>
+          <t>S4</t>
         </is>
       </c>
       <c r="E60" s="11" t="inlineStr">
         <is>
-          <t>hệ số 19 suy từ cột tổng (2,581.50 ÷ 135.90) — xem PDF tr.119</t>
+          <t>hệ số 2 suy từ cột tổng (907.20 ÷ 453.60) — xem PDF tr.112</t>
         </is>
       </c>
       <c r="F60" t="inlineStr"/>
@@ -34136,7 +34142,7 @@
         <v>58</v>
       </c>
       <c r="B61" t="n">
-        <v>338</v>
+        <v>337</v>
       </c>
       <c r="C61" t="inlineStr">
         <is>
@@ -34145,12 +34151,12 @@
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>G2</t>
+          <t>G1</t>
         </is>
       </c>
       <c r="E61" s="11" t="inlineStr">
         <is>
-          <t>hệ số 19 suy từ cột tổng (4,016.50 ÷ 211.40) — xem PDF tr.119</t>
+          <t>hệ số 19 suy từ cột tổng (2,581.50 ÷ 135.90) — xem PDF tr.119</t>
         </is>
       </c>
       <c r="F61" t="inlineStr"/>
@@ -34163,7 +34169,7 @@
         <v>59</v>
       </c>
       <c r="B62" t="n">
-        <v>339</v>
+        <v>338</v>
       </c>
       <c r="C62" t="inlineStr">
         <is>
@@ -34172,12 +34178,12 @@
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>G3</t>
+          <t>G2</t>
         </is>
       </c>
       <c r="E62" s="11" t="inlineStr">
         <is>
-          <t>hệ số 19 suy từ cột tổng (2,209.40 ÷ 116.30) — xem PDF tr.119</t>
+          <t>hệ số 19 suy từ cột tổng (4,016.50 ÷ 211.40) — xem PDF tr.119</t>
         </is>
       </c>
       <c r="F62" t="inlineStr"/>
@@ -34190,7 +34196,7 @@
         <v>60</v>
       </c>
       <c r="B63" t="n">
-        <v>340</v>
+        <v>339</v>
       </c>
       <c r="C63" t="inlineStr">
         <is>
@@ -34199,12 +34205,12 @@
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>G4A</t>
+          <t>G3</t>
         </is>
       </c>
       <c r="E63" s="11" t="inlineStr">
         <is>
-          <t>khối lượng 1 cấu kiện trống, = dài × SL × kg/m; hệ số 19 = tổng ÷ khối lượng — Σ bảng sau sửa khớp tổng bản vẽ — xem PDF tr.119</t>
+          <t>hệ số 19 suy từ cột tổng (2,209.40 ÷ 116.30) — xem PDF tr.119</t>
         </is>
       </c>
       <c r="F63" t="inlineStr"/>
@@ -34217,7 +34223,7 @@
         <v>61</v>
       </c>
       <c r="B64" t="n">
-        <v>341</v>
+        <v>340</v>
       </c>
       <c r="C64" t="inlineStr">
         <is>
@@ -34226,12 +34232,12 @@
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>G4B</t>
+          <t>G4A</t>
         </is>
       </c>
       <c r="E64" s="11" t="inlineStr">
         <is>
-          <t>hệ số 19 suy từ cột tổng (85.10 ÷ dài × SL × kg/m 4.48) — ô số cấu kiện gộp/không đọc được — xem PDF tr.119</t>
+          <t>khối lượng 1 cấu kiện trống, = dài × SL × kg/m; hệ số 19 = tổng ÷ khối lượng — Σ bảng sau sửa khớp tổng bản vẽ — xem PDF tr.119</t>
         </is>
       </c>
       <c r="F64" t="inlineStr"/>
@@ -34244,7 +34250,7 @@
         <v>62</v>
       </c>
       <c r="B65" t="n">
-        <v>342</v>
+        <v>341</v>
       </c>
       <c r="C65" t="inlineStr">
         <is>
@@ -34253,12 +34259,12 @@
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>G4C</t>
+          <t>G4B</t>
         </is>
       </c>
       <c r="E65" s="11" t="inlineStr">
         <is>
-          <t>hệ số 19 suy từ cột tổng (139.10 ÷ dài × SL × kg/m 7.32) — ô số cấu kiện gộp/không đọc được — xem PDF tr.119</t>
+          <t>hệ số 19 suy từ cột tổng (85.10 ÷ dài × SL × kg/m 4.48) — ô số cấu kiện gộp/không đọc được — xem PDF tr.119</t>
         </is>
       </c>
       <c r="F65" t="inlineStr"/>
@@ -34271,7 +34277,7 @@
         <v>63</v>
       </c>
       <c r="B66" t="n">
-        <v>349</v>
+        <v>342</v>
       </c>
       <c r="C66" t="inlineStr">
         <is>
@@ -34280,12 +34286,12 @@
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>G5</t>
+          <t>G4C</t>
         </is>
       </c>
       <c r="E66" s="11" t="inlineStr">
         <is>
-          <t>hệ số 19 suy từ cột tổng (2,581.50 ÷ 135.90) — xem PDF tr.119</t>
+          <t>hệ số 19 suy từ cột tổng (139.10 ÷ dài × SL × kg/m 7.32) — ô số cấu kiện gộp/không đọc được — xem PDF tr.119</t>
         </is>
       </c>
       <c r="F66" t="inlineStr"/>
@@ -34298,7 +34304,7 @@
         <v>64</v>
       </c>
       <c r="B67" t="n">
-        <v>350</v>
+        <v>349</v>
       </c>
       <c r="C67" t="inlineStr">
         <is>
@@ -34307,12 +34313,12 @@
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>G6</t>
+          <t>G5</t>
         </is>
       </c>
       <c r="E67" s="11" t="inlineStr">
         <is>
-          <t>hệ số 19 suy từ cột tổng (3,898.30 ÷ 205.20) — xem PDF tr.119</t>
+          <t>hệ số 19 suy từ cột tổng (2,581.50 ÷ 135.90) — xem PDF tr.119</t>
         </is>
       </c>
       <c r="F67" t="inlineStr"/>
@@ -34325,7 +34331,7 @@
         <v>65</v>
       </c>
       <c r="B68" t="n">
-        <v>351</v>
+        <v>350</v>
       </c>
       <c r="C68" t="inlineStr">
         <is>
@@ -34334,12 +34340,12 @@
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>G7</t>
+          <t>G6</t>
         </is>
       </c>
       <c r="E68" s="11" t="inlineStr">
         <is>
-          <t>hệ số 19 suy từ cột tổng (1,292.30 ÷ 68.00) — xem PDF tr.119</t>
+          <t>hệ số 19 suy từ cột tổng (3,898.30 ÷ 205.20) — xem PDF tr.119</t>
         </is>
       </c>
       <c r="F68" t="inlineStr"/>
@@ -34352,7 +34358,7 @@
         <v>66</v>
       </c>
       <c r="B69" t="n">
-        <v>352</v>
+        <v>351</v>
       </c>
       <c r="C69" t="inlineStr">
         <is>
@@ -34361,12 +34367,12 @@
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>G7A</t>
+          <t>G7</t>
         </is>
       </c>
       <c r="E69" s="11" t="inlineStr">
         <is>
-          <t>hệ số 19 suy từ cột tổng (2,274.30 ÷ 119.70) — xem PDF tr.119</t>
+          <t>hệ số 19 suy từ cột tổng (1,292.30 ÷ 68.00) — xem PDF tr.119</t>
         </is>
       </c>
       <c r="F69" t="inlineStr"/>
@@ -34379,7 +34385,7 @@
         <v>67</v>
       </c>
       <c r="B70" t="n">
-        <v>353</v>
+        <v>352</v>
       </c>
       <c r="C70" t="inlineStr">
         <is>
@@ -34388,12 +34394,12 @@
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>G8A</t>
+          <t>G7A</t>
         </is>
       </c>
       <c r="E70" s="11" t="inlineStr">
         <is>
-          <t>hệ số 19 suy từ cột tổng (57.00 ÷ 3.00) — xem PDF tr.119</t>
+          <t>hệ số 19 suy từ cột tổng (2,274.30 ÷ 119.70) — xem PDF tr.119</t>
         </is>
       </c>
       <c r="F70" t="inlineStr"/>
@@ -34406,7 +34412,7 @@
         <v>68</v>
       </c>
       <c r="B71" t="n">
-        <v>354</v>
+        <v>353</v>
       </c>
       <c r="C71" t="inlineStr">
         <is>
@@ -34415,12 +34421,12 @@
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>G8B</t>
+          <t>G8A</t>
         </is>
       </c>
       <c r="E71" s="11" t="inlineStr">
         <is>
-          <t>hệ số 19 suy từ cột tổng (67.10 ÷ dài × SL × kg/m 3.53) — ô số cấu kiện gộp/không đọc được — xem PDF tr.119</t>
+          <t>hệ số 19 suy từ cột tổng (57.00 ÷ 3.00) — xem PDF tr.119</t>
         </is>
       </c>
       <c r="F71" t="inlineStr"/>
@@ -34433,7 +34439,7 @@
         <v>69</v>
       </c>
       <c r="B72" t="n">
-        <v>355</v>
+        <v>354</v>
       </c>
       <c r="C72" t="inlineStr">
         <is>
@@ -34442,12 +34448,12 @@
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t>G8C</t>
+          <t>G8B</t>
         </is>
       </c>
       <c r="E72" s="11" t="inlineStr">
         <is>
-          <t>hệ số 19 suy từ cột tổng (91.50 ÷ dài × SL × kg/m 4.81) — ô số cấu kiện gộp/không đọc được — xem PDF tr.119</t>
+          <t>hệ số 19 suy từ cột tổng (67.10 ÷ dài × SL × kg/m 3.53) — ô số cấu kiện gộp/không đọc được — xem PDF tr.119</t>
         </is>
       </c>
       <c r="F72" t="inlineStr"/>
@@ -34460,7 +34466,7 @@
         <v>70</v>
       </c>
       <c r="B73" t="n">
-        <v>360</v>
+        <v>355</v>
       </c>
       <c r="C73" t="inlineStr">
         <is>
@@ -34469,12 +34475,12 @@
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t>G8A</t>
+          <t>G8C</t>
         </is>
       </c>
       <c r="E73" s="11" t="inlineStr">
         <is>
-          <t>OCR đọc SL = 6, phép tính bản vẽ cho 9 (khối lượng ghi ÷ dài ÷ kg/m) — Σ bảng sau sửa khớp tổng bản vẽ — xem PDF tr.119</t>
+          <t>hệ số 19 suy từ cột tổng (91.50 ÷ dài × SL × kg/m 4.81) — ô số cấu kiện gộp/không đọc được — xem PDF tr.119</t>
         </is>
       </c>
       <c r="F73" t="inlineStr"/>
@@ -34487,21 +34493,21 @@
         <v>71</v>
       </c>
       <c r="B74" t="n">
-        <v>363</v>
+        <v>360</v>
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>Khe co giãn</t>
+          <t>Gờ lan can BTCT</t>
         </is>
       </c>
       <c r="D74" t="inlineStr">
         <is>
-          <t>K1</t>
+          <t>G8A</t>
         </is>
       </c>
       <c r="E74" s="11" t="inlineStr">
         <is>
-          <t>hệ số 2 suy từ cột tổng (586.67 ÷ 293.33) — xem PDF tr.121</t>
+          <t>OCR đọc SL = 6, phép tính bản vẽ cho 9 (khối lượng ghi ÷ dài ÷ kg/m) — Σ bảng sau sửa khớp tổng bản vẽ — xem PDF tr.119</t>
         </is>
       </c>
       <c r="F74" t="inlineStr"/>
@@ -34514,7 +34520,7 @@
         <v>72</v>
       </c>
       <c r="B75" t="n">
-        <v>364</v>
+        <v>363</v>
       </c>
       <c r="C75" t="inlineStr">
         <is>
@@ -34523,12 +34529,12 @@
       </c>
       <c r="D75" t="inlineStr">
         <is>
-          <t>K2</t>
+          <t>K1</t>
         </is>
       </c>
       <c r="E75" s="11" t="inlineStr">
         <is>
-          <t>hệ số 2 suy từ cột tổng (521.99 ÷ 260.99) — xem PDF tr.121</t>
+          <t>hệ số 2 suy từ cột tổng (586.67 ÷ 293.33) — xem PDF tr.121</t>
         </is>
       </c>
       <c r="F75" t="inlineStr"/>
@@ -34541,7 +34547,7 @@
         <v>73</v>
       </c>
       <c r="B76" t="n">
-        <v>365</v>
+        <v>364</v>
       </c>
       <c r="C76" t="inlineStr">
         <is>
@@ -34550,12 +34556,12 @@
       </c>
       <c r="D76" t="inlineStr">
         <is>
-          <t>K3</t>
+          <t>K2</t>
         </is>
       </c>
       <c r="E76" s="11" t="inlineStr">
         <is>
-          <t>hệ số 2 suy từ cột tổng (251.14 ÷ 125.57) — xem PDF tr.121</t>
+          <t>hệ số 2 suy từ cột tổng (521.99 ÷ 260.99) — xem PDF tr.121</t>
         </is>
       </c>
       <c r="F76" t="inlineStr"/>
@@ -34563,6 +34569,33 @@
       <c r="H76" t="inlineStr"/>
       <c r="I76" t="inlineStr"/>
     </row>
+    <row r="77">
+      <c r="A77" t="n">
+        <v>74</v>
+      </c>
+      <c r="B77" t="n">
+        <v>365</v>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>Khe co giãn</t>
+        </is>
+      </c>
+      <c r="D77" t="inlineStr">
+        <is>
+          <t>K3</t>
+        </is>
+      </c>
+      <c r="E77" s="11" t="inlineStr">
+        <is>
+          <t>hệ số 2 suy từ cột tổng (251.14 ÷ 125.57) — xem PDF tr.121</t>
+        </is>
+      </c>
+      <c r="F77" t="inlineStr"/>
+      <c r="G77" t="inlineStr"/>
+      <c r="H77" t="inlineStr"/>
+      <c r="I77" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
data(km19): S1B3 dùng bảng thép như S1B1 — chủ dự án xác nhận; sinh lại bộ file cắt thép
- Chủ dự án xác nhận 11/10/2026: 2 S1B1 + 3 S1B2 + 1 S1B3 + 9 S1G, S1B3 dùng bảng thép S1B1 (tr.88).
  Cấu hình 'da_xac_nhan' bỏ mục "số cấu kiện cần xác nhận" khỏi NGHI_VAN; các dòng sửa OCR của bảng dầm vẫn
  để soát.
- Bộ file cắt thép sinh lại từ BBS có dòng S1B3 riêng: 20.311 cây 11,7 m, 0 thanh chưa lập kế hoạch,
  đề-xê chung 1,79% (không đổi số cây); Ø16 FEASIBLE (60 s/Ø), các Ø khác OPTIMAL.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_013xu17UUNVqCoEvpVUxkPSc
</commit_message>
<xml_diff>
--- a/examples/HO_SO_CAU_KM19_529/02_XUONG_TIEN_CHE_COT_THEP/04_Thong_Ke_Thep_Chi_Tiet_BBS_396_Dong.xlsx
+++ b/examples/HO_SO_CAU_KM19_529/02_XUONG_TIEN_CHE_COT_THEP/04_Thong_Ke_Thep_Chi_Tiet_BBS_396_Dong.xlsx
@@ -19747,7 +19747,7 @@
       </c>
       <c r="C266" s="5" t="inlineStr">
         <is>
-          <t>Dầm S1B3 (dùng bảng thép S1B1) (tr.88)</t>
+          <t>Dầm S1B3 (bảng thép như S1B1) (tr.88)</t>
         </is>
       </c>
       <c r="D266" s="5" t="inlineStr">
@@ -19823,7 +19823,7 @@
       </c>
       <c r="C267" s="5" t="inlineStr">
         <is>
-          <t>Dầm S1B3 (dùng bảng thép S1B1) (tr.88)</t>
+          <t>Dầm S1B3 (bảng thép như S1B1) (tr.88)</t>
         </is>
       </c>
       <c r="D267" s="5" t="inlineStr">
@@ -19899,7 +19899,7 @@
       </c>
       <c r="C268" s="5" t="inlineStr">
         <is>
-          <t>Dầm S1B3 (dùng bảng thép S1B1) (tr.88)</t>
+          <t>Dầm S1B3 (bảng thép như S1B1) (tr.88)</t>
         </is>
       </c>
       <c r="D268" s="5" t="inlineStr">
@@ -19975,7 +19975,7 @@
       </c>
       <c r="C269" s="5" t="inlineStr">
         <is>
-          <t>Dầm S1B3 (dùng bảng thép S1B1) (tr.88)</t>
+          <t>Dầm S1B3 (bảng thép như S1B1) (tr.88)</t>
         </is>
       </c>
       <c r="D269" s="5" t="inlineStr">
@@ -20051,7 +20051,7 @@
       </c>
       <c r="C270" s="5" t="inlineStr">
         <is>
-          <t>Dầm S1B3 (dùng bảng thép S1B1) (tr.88)</t>
+          <t>Dầm S1B3 (bảng thép như S1B1) (tr.88)</t>
         </is>
       </c>
       <c r="D270" s="5" t="inlineStr">
@@ -20127,7 +20127,7 @@
       </c>
       <c r="C271" s="5" t="inlineStr">
         <is>
-          <t>Dầm S1B3 (dùng bảng thép S1B1) (tr.88)</t>
+          <t>Dầm S1B3 (bảng thép như S1B1) (tr.88)</t>
         </is>
       </c>
       <c r="D271" s="5" t="inlineStr">
@@ -20203,7 +20203,7 @@
       </c>
       <c r="C272" s="5" t="inlineStr">
         <is>
-          <t>Dầm S1B3 (dùng bảng thép S1B1) (tr.88)</t>
+          <t>Dầm S1B3 (bảng thép như S1B1) (tr.88)</t>
         </is>
       </c>
       <c r="D272" s="5" t="inlineStr">
@@ -20279,7 +20279,7 @@
       </c>
       <c r="C273" s="5" t="inlineStr">
         <is>
-          <t>Dầm S1B3 (dùng bảng thép S1B1) (tr.88)</t>
+          <t>Dầm S1B3 (bảng thép như S1B1) (tr.88)</t>
         </is>
       </c>
       <c r="D273" s="5" t="inlineStr">
@@ -20355,7 +20355,7 @@
       </c>
       <c r="C274" s="5" t="inlineStr">
         <is>
-          <t>Dầm S1B3 (dùng bảng thép S1B1) (tr.88)</t>
+          <t>Dầm S1B3 (bảng thép như S1B1) (tr.88)</t>
         </is>
       </c>
       <c r="D274" s="5" t="inlineStr">
@@ -20431,7 +20431,7 @@
       </c>
       <c r="C275" s="5" t="inlineStr">
         <is>
-          <t>Dầm S1B3 (dùng bảng thép S1B1) (tr.88)</t>
+          <t>Dầm S1B3 (bảng thép như S1B1) (tr.88)</t>
         </is>
       </c>
       <c r="D275" s="5" t="inlineStr">
@@ -20507,7 +20507,7 @@
       </c>
       <c r="C276" s="5" t="inlineStr">
         <is>
-          <t>Dầm S1B3 (dùng bảng thép S1B1) (tr.88)</t>
+          <t>Dầm S1B3 (bảng thép như S1B1) (tr.88)</t>
         </is>
       </c>
       <c r="D276" s="5" t="inlineStr">
@@ -20583,7 +20583,7 @@
       </c>
       <c r="C277" s="5" t="inlineStr">
         <is>
-          <t>Dầm S1B3 (dùng bảng thép S1B1) (tr.88)</t>
+          <t>Dầm S1B3 (bảng thép như S1B1) (tr.88)</t>
         </is>
       </c>
       <c r="D277" s="5" t="inlineStr">
@@ -20659,7 +20659,7 @@
       </c>
       <c r="C278" s="5" t="inlineStr">
         <is>
-          <t>Dầm S1B3 (dùng bảng thép S1B1) (tr.88)</t>
+          <t>Dầm S1B3 (bảng thép như S1B1) (tr.88)</t>
         </is>
       </c>
       <c r="D278" s="5" t="inlineStr">
@@ -20735,7 +20735,7 @@
       </c>
       <c r="C279" s="5" t="inlineStr">
         <is>
-          <t>Dầm S1B3 (dùng bảng thép S1B1) (tr.88)</t>
+          <t>Dầm S1B3 (bảng thép như S1B1) (tr.88)</t>
         </is>
       </c>
       <c r="D279" s="5" t="inlineStr">
@@ -20811,7 +20811,7 @@
       </c>
       <c r="C280" s="5" t="inlineStr">
         <is>
-          <t>Dầm S1B3 (dùng bảng thép S1B1) (tr.88)</t>
+          <t>Dầm S1B3 (bảng thép như S1B1) (tr.88)</t>
         </is>
       </c>
       <c r="D280" s="5" t="inlineStr">
@@ -20887,7 +20887,7 @@
       </c>
       <c r="C281" s="5" t="inlineStr">
         <is>
-          <t>Dầm S1B3 (dùng bảng thép S1B1) (tr.88)</t>
+          <t>Dầm S1B3 (bảng thép như S1B1) (tr.88)</t>
         </is>
       </c>
       <c r="D281" s="5" t="inlineStr">
@@ -20963,7 +20963,7 @@
       </c>
       <c r="C282" s="5" t="inlineStr">
         <is>
-          <t>Dầm S1B3 (dùng bảng thép S1B1) (tr.88)</t>
+          <t>Dầm S1B3 (bảng thép như S1B1) (tr.88)</t>
         </is>
       </c>
       <c r="D282" s="5" t="inlineStr">
@@ -21039,7 +21039,7 @@
       </c>
       <c r="C283" s="5" t="inlineStr">
         <is>
-          <t>Dầm S1B3 (dùng bảng thép S1B1) (tr.88)</t>
+          <t>Dầm S1B3 (bảng thép như S1B1) (tr.88)</t>
         </is>
       </c>
       <c r="D283" s="5" t="inlineStr">
@@ -21115,7 +21115,7 @@
       </c>
       <c r="C284" s="5" t="inlineStr">
         <is>
-          <t>Dầm S1B3 (dùng bảng thép S1B1) (tr.88)</t>
+          <t>Dầm S1B3 (bảng thép như S1B1) (tr.88)</t>
         </is>
       </c>
       <c r="D284" s="5" t="inlineStr">
@@ -21191,7 +21191,7 @@
       </c>
       <c r="C285" s="5" t="inlineStr">
         <is>
-          <t>Dầm S1B3 (dùng bảng thép S1B1) (tr.88)</t>
+          <t>Dầm S1B3 (bảng thép như S1B1) (tr.88)</t>
         </is>
       </c>
       <c r="D285" s="5" t="inlineStr">
@@ -21267,7 +21267,7 @@
       </c>
       <c r="C286" s="5" t="inlineStr">
         <is>
-          <t>Dầm S1B3 (dùng bảng thép S1B1) (tr.88)</t>
+          <t>Dầm S1B3 (bảng thép như S1B1) (tr.88)</t>
         </is>
       </c>
       <c r="D286" s="5" t="inlineStr">
@@ -21343,7 +21343,7 @@
       </c>
       <c r="C287" s="5" t="inlineStr">
         <is>
-          <t>Dầm S1B3 (dùng bảng thép S1B1) (tr.88)</t>
+          <t>Dầm S1B3 (bảng thép như S1B1) (tr.88)</t>
         </is>
       </c>
       <c r="D287" s="5" t="inlineStr">
@@ -21419,7 +21419,7 @@
       </c>
       <c r="C288" s="5" t="inlineStr">
         <is>
-          <t>Dầm S1B3 (dùng bảng thép S1B1) (tr.88)</t>
+          <t>Dầm S1B3 (bảng thép như S1B1) (tr.88)</t>
         </is>
       </c>
       <c r="D288" s="5" t="inlineStr">
@@ -33879,7 +33879,7 @@
       </c>
       <c r="I10" s="10" t="inlineStr">
         <is>
-          <t>Số phiến theo chủ dự án 11/10/2026: 2 S1B1 + 3 S1B2 + 1 S1B3 + 9 S1G (khớp sơ đồ bố trí nhịp tr.75). Hồ sơ không có bảng thép riêng cho S1B3 (tr.86–94 chỉ có S1B1, S1B2, S1G) — tạm dùng bảng S1B1 tr.88; tổng 89.690,31 kg khớp tr.175 chỉ khi S1B3 = S1B1. Đối chiếu PDF bản vẽ S1B3.</t>
+          <t>Chủ dự án xác nhận 11/10/2026: 2 S1B1 + 3 S1B2 + 1 S1B3 + 9 S1G (khớp sơ đồ bố trí nhịp tr.75); S1B3 dùng bảng thép giống S1B1 (tr.88). Tổng 89.690,31 kg khớp bảng tổng hợp tr.175 (77,743 + 11,947 t).</t>
         </is>
       </c>
     </row>
@@ -34162,7 +34162,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I79"/>
+  <dimension ref="A1:I78"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -34450,11 +34450,19 @@
       <c r="D11" t="inlineStr"/>
       <c r="E11" s="11" t="inlineStr">
         <is>
-          <t>Số cấu kiện cần xác nhận: Số phiến theo chủ dự án 11/10/2026: 2 S1B1 + 3 S1B2 + 1 S1B3 + 9 S1G (khớp sơ đồ bố trí nhịp tr.75). Hồ sơ không có bảng thép riêng cho S1B3 (tr.86–94 chỉ có S1B1, S1B2, S1G) — tạm dùng bảng S1B1 tr.88; tổng 89.690,31 kg khớp tr.175 chỉ khi S1B3 = S1B1. Đối chiếu PDF bản vẽ S1B3.</t>
-        </is>
-      </c>
-      <c r="F11" t="inlineStr"/>
-      <c r="G11" t="inlineStr"/>
+          <t>THAY THEO BẢN VẼ: BBS cũ 361.596,10 kg; bản vẽ 89.690,31 kg</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>361.596,10 kg</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>89.690,31 kg</t>
+        </is>
+      </c>
       <c r="H11" t="inlineStr">
         <is>
           <t>tr.88, tr.91, tr.88, tr.94</t>
@@ -34469,30 +34477,30 @@
       <c r="B12" t="inlineStr"/>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Dầm chủ Super-T (15 phiến L=38.2m)</t>
-        </is>
-      </c>
-      <c r="D12" t="inlineStr"/>
+          <t>Dầm ngang (Diaphragm)</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>16</t>
+        </is>
+      </c>
       <c r="E12" s="11" t="inlineStr">
         <is>
-          <t>THAY THEO BẢN VẼ: BBS cũ 361.596,10 kg; bản vẽ 89.690,31 kg</t>
+          <t>Dòng BBS cũ sai rõ ràng (Ø không phải thép thanh hoặc dài &lt; 50 mm) — đã loại</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>361.596,10 kg</t>
+          <t>Ø128 L=0.002 m × 525 × 1, 106.18 kg/m = 111,49 kg</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>89.690,31 kg</t>
-        </is>
-      </c>
-      <c r="H12" t="inlineStr">
-        <is>
-          <t>tr.88, tr.91, tr.88, tr.94</t>
-        </is>
-      </c>
+          <t>đã loại</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr"/>
       <c r="I12" t="inlineStr"/>
     </row>
     <row r="13">
@@ -34507,7 +34515,7 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>16</t>
+          <t>20</t>
         </is>
       </c>
       <c r="E13" s="11" t="inlineStr">
@@ -34517,7 +34525,7 @@
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>Ø128 L=0.002 m × 525 × 1, 106.18 kg/m = 111,49 kg</t>
+          <t>Ø32 L=0.002 m × 1450 × 1, 114.61 kg/m = 332,37 kg</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
@@ -34540,7 +34548,7 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>20</t>
+          <t>16</t>
         </is>
       </c>
       <c r="E14" s="11" t="inlineStr">
@@ -34550,7 +34558,7 @@
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>Ø32 L=0.002 m × 1450 × 1, 114.61 kg/m = 332,37 kg</t>
+          <t>Ø112 L=0.002 m × 1390 × 1, 245.97 kg/m = 683,80 kg</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
@@ -34583,7 +34591,7 @@
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>Ø112 L=0.002 m × 1390 × 1, 245.97 kg/m = 683,80 kg</t>
+          <t>Ø32 L=0.002 m × 1140 × 1, 57.64 kg/m = 131,42 kg</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
@@ -34616,7 +34624,7 @@
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>Ø32 L=0.002 m × 1140 × 1, 57.64 kg/m = 131,42 kg</t>
+          <t>Ø64 L=0.002 m × 3262 × 1, 329.85 kg/m = 2.151,94 kg</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
@@ -34649,7 +34657,7 @@
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>Ø64 L=0.002 m × 3262 × 1, 329.85 kg/m = 2.151,94 kg</t>
+          <t>Ø16 L=0.002 m × 2642 × 1, 66.79 kg/m = 352,92 kg</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
@@ -34670,27 +34678,27 @@
           <t>Dầm ngang (Diaphragm)</t>
         </is>
       </c>
-      <c r="D18" t="inlineStr">
-        <is>
-          <t>16</t>
-        </is>
-      </c>
+      <c r="D18" t="inlineStr"/>
       <c r="E18" s="11" t="inlineStr">
         <is>
-          <t>Dòng BBS cũ sai rõ ràng (Ø không phải thép thanh hoặc dài &lt; 50 mm) — đã loại</t>
+          <t>THAY THEO BẢN VẼ: BBS cũ 0,00 kg (+ 6 dòng lỗi 3.763,93 kg); bản vẽ 2.763,12 kg</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>Ø16 L=0.002 m × 2642 × 1, 66.79 kg/m = 352,92 kg</t>
+          <t>3.763,93 kg</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>đã loại</t>
-        </is>
-      </c>
-      <c r="H18" t="inlineStr"/>
+          <t>2.763,12 kg</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>tr.96</t>
+        </is>
+      </c>
       <c r="I18" t="inlineStr"/>
     </row>
     <row r="19">
@@ -34700,30 +34708,30 @@
       <c r="B19" t="inlineStr"/>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Dầm ngang (Diaphragm)</t>
-        </is>
-      </c>
-      <c r="D19" t="inlineStr"/>
+          <t>Bản liên tục nhiệt (Link Slab)</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>18</t>
+        </is>
+      </c>
       <c r="E19" s="11" t="inlineStr">
         <is>
-          <t>THAY THEO BẢN VẼ: BBS cũ 0,00 kg (+ 6 dòng lỗi 3.763,93 kg); bản vẽ 2.763,12 kg</t>
+          <t>Dòng BBS cũ sai rõ ràng (Ø không phải thép thanh hoặc dài &lt; 50 mm) — đã loại</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>3.763,93 kg</t>
+          <t>Ø54 L=0.002 m × 13135 × 1, 1418.58 kg/m = 37.266,10 kg</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>2.763,12 kg</t>
-        </is>
-      </c>
-      <c r="H19" t="inlineStr">
-        <is>
-          <t>tr.96</t>
-        </is>
-      </c>
+          <t>đã loại</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr"/>
       <c r="I19" t="inlineStr"/>
     </row>
     <row r="20">
@@ -34738,7 +34746,7 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>18</t>
+          <t>25</t>
         </is>
       </c>
       <c r="E20" s="11" t="inlineStr">
@@ -34748,7 +34756,7 @@
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>Ø54 L=0.002 m × 13135 × 1, 1418.58 kg/m = 37.266,10 kg</t>
+          <t>Ø168 L=0.004 m × 3920 × 1, 2535.46 kg/m = 39.756,01 kg</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
@@ -34771,7 +34779,7 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>25</t>
+          <t>10</t>
         </is>
       </c>
       <c r="E21" s="11" t="inlineStr">
@@ -34781,7 +34789,7 @@
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>Ø168 L=0.004 m × 3920 × 1, 2535.46 kg/m = 39.756,01 kg</t>
+          <t>Ø260 L=0.001 m × 320 × 1, 51.33 kg/m = 16,43 kg</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
@@ -34804,7 +34812,7 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>18</t>
         </is>
       </c>
       <c r="E22" s="11" t="inlineStr">
@@ -34814,7 +34822,7 @@
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>Ø260 L=0.001 m × 320 × 1, 51.33 kg/m = 16,43 kg</t>
+          <t>Ø108 L=0.002 m × 2100 × 1, 453.6 kg/m = 1.905,12 kg</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
@@ -34835,27 +34843,27 @@
           <t>Bản liên tục nhiệt (Link Slab)</t>
         </is>
       </c>
-      <c r="D23" t="inlineStr">
-        <is>
-          <t>18</t>
-        </is>
-      </c>
+      <c r="D23" t="inlineStr"/>
       <c r="E23" s="11" t="inlineStr">
         <is>
-          <t>Dòng BBS cũ sai rõ ràng (Ø không phải thép thanh hoặc dài &lt; 50 mm) — đã loại</t>
+          <t>THAY THEO BẢN VẼ: BBS cũ 0,00 kg (+ 4 dòng lỗi 78.943,65 kg); bản vẽ 8.917,94 kg</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>Ø108 L=0.002 m × 2100 × 1, 453.6 kg/m = 1.905,12 kg</t>
+          <t>78.943,65 kg</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>đã loại</t>
-        </is>
-      </c>
-      <c r="H23" t="inlineStr"/>
+          <t>8.917,94 kg</t>
+        </is>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>tr.112</t>
+        </is>
+      </c>
       <c r="I23" t="inlineStr"/>
     </row>
     <row r="24">
@@ -34865,28 +34873,28 @@
       <c r="B24" t="inlineStr"/>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Bản liên tục nhiệt (Link Slab)</t>
+          <t>Gờ lan can BTCT</t>
         </is>
       </c>
       <c r="D24" t="inlineStr"/>
       <c r="E24" s="11" t="inlineStr">
         <is>
-          <t>THAY THEO BẢN VẼ: BBS cũ 0,00 kg (+ 4 dòng lỗi 78.943,65 kg); bản vẽ 8.917,94 kg</t>
+          <t>THAY THEO BẢN VẼ: BBS cũ 1.719,70 kg; bản vẽ 20.069,02 kg</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>78.943,65 kg</t>
+          <t>1.719,70 kg</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>8.917,94 kg</t>
+          <t>20.069,02 kg</t>
         </is>
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>tr.112</t>
+          <t>tr.119</t>
         </is>
       </c>
       <c r="I24" t="inlineStr"/>
@@ -34898,28 +34906,28 @@
       <c r="B25" t="inlineStr"/>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Gờ lan can BTCT</t>
+          <t>Khe co giãn</t>
         </is>
       </c>
       <c r="D25" t="inlineStr"/>
       <c r="E25" s="11" t="inlineStr">
         <is>
-          <t>THAY THEO BẢN VẼ: BBS cũ 1.719,70 kg; bản vẽ 20.069,02 kg</t>
+          <t>THAY THEO BẢN VẼ: BBS cũ 0,00 kg; bản vẽ 1.359,80 kg</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>1.719,70 kg</t>
+          <t>0,00 kg</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>20.069,02 kg</t>
+          <t>1.359,80 kg</t>
         </is>
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>tr.119</t>
+          <t>tr.121</t>
         </is>
       </c>
       <c r="I25" t="inlineStr"/>
@@ -34931,28 +34939,28 @@
       <c r="B26" t="inlineStr"/>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Khe co giãn</t>
+          <t>Cọc khoan nhồi D1200 (26 cọc L=872m)</t>
         </is>
       </c>
       <c r="D26" t="inlineStr"/>
       <c r="E26" s="11" t="inlineStr">
         <is>
-          <t>THAY THEO BẢN VẼ: BBS cũ 0,00 kg; bản vẽ 1.359,80 kg</t>
+          <t>Tổng các trang chi tiết 108.461,59 kg ≠ bảng tổng hợp tr.175 108.884,00 kg (lệch 422,41 kg). Tr.175: D&lt;=10 10,451 t và D&gt;18 97,451 t khớp đúng 3/7/8/8 cọc; nhóm 10&lt;D&lt;=18 ghi 0,982 t nhưng các trang cọc chỉ có 0,559 t — xem PDF tr.175.</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>0,00 kg</t>
+          <t>108.461,59 kg</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>1.359,80 kg</t>
+          <t>108.884,00 kg</t>
         </is>
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>tr.121</t>
+          <t>tr.175</t>
         </is>
       </c>
       <c r="I26" t="inlineStr"/>
@@ -34970,22 +34978,14 @@
       <c r="D27" t="inlineStr"/>
       <c r="E27" s="11" t="inlineStr">
         <is>
-          <t>Tổng các trang chi tiết 108.461,59 kg ≠ bảng tổng hợp tr.175 108.884,00 kg (lệch 422,41 kg). Tr.175: D&lt;=10 10,451 t và D&gt;18 97,451 t khớp đúng 3/7/8/8 cọc; nhóm 10&lt;D&lt;=18 ghi 0,982 t nhưng các trang cọc chỉ có 0,559 t — xem PDF tr.175.</t>
-        </is>
-      </c>
-      <c r="F27" t="inlineStr">
-        <is>
-          <t>108.461,59 kg</t>
-        </is>
-      </c>
-      <c r="G27" t="inlineStr">
-        <is>
-          <t>108.884,00 kg</t>
-        </is>
-      </c>
+          <t>Số cấu kiện cần xác nhận: Số cọc 3/7/8/8 khớp bảng tổng hợp tr.175 (thép D&lt;=10, D&gt;18 và vữa lấp lòng 14,43 m³ = 3×0,34 + 7×0,59 + 8×0,66 + 8×0,50).</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr"/>
+      <c r="G27" t="inlineStr"/>
       <c r="H27" t="inlineStr">
         <is>
-          <t>tr.175</t>
+          <t>tr.64, tr.66, tr.68, tr.70</t>
         </is>
       </c>
       <c r="I27" t="inlineStr"/>
@@ -35003,11 +35003,19 @@
       <c r="D28" t="inlineStr"/>
       <c r="E28" s="11" t="inlineStr">
         <is>
-          <t>Số cấu kiện cần xác nhận: Số cọc 3/7/8/8 khớp bảng tổng hợp tr.175 (thép D&lt;=10, D&gt;18 và vữa lấp lòng 14,43 m³ = 3×0,34 + 7×0,59 + 8×0,66 + 8×0,50).</t>
-        </is>
-      </c>
-      <c r="F28" t="inlineStr"/>
-      <c r="G28" t="inlineStr"/>
+          <t>THAY THEO BẢN VẼ: BBS cũ 108.765,99 kg; bản vẽ 108.461,59 kg</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>108.765,99 kg</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>108.461,59 kg</t>
+        </is>
+      </c>
       <c r="H28" t="inlineStr">
         <is>
           <t>tr.64, tr.66, tr.68, tr.70</t>
@@ -35019,33 +35027,27 @@
       <c r="A29" t="n">
         <v>26</v>
       </c>
-      <c r="B29" t="inlineStr"/>
+      <c r="B29" t="n">
+        <v>44</v>
+      </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Cọc khoan nhồi D1200 (26 cọc L=872m)</t>
-        </is>
-      </c>
-      <c r="D29" t="inlineStr"/>
+          <t>Mố M1</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>B1</t>
+        </is>
+      </c>
       <c r="E29" s="11" t="inlineStr">
         <is>
-          <t>THAY THEO BẢN VẼ: BBS cũ 108.765,99 kg; bản vẽ 108.461,59 kg</t>
-        </is>
-      </c>
-      <c r="F29" t="inlineStr">
-        <is>
-          <t>108.765,99 kg</t>
-        </is>
-      </c>
-      <c r="G29" t="inlineStr">
-        <is>
-          <t>108.461,59 kg</t>
-        </is>
-      </c>
-      <c r="H29" t="inlineStr">
-        <is>
-          <t>tr.64, tr.66, tr.68, tr.70</t>
-        </is>
-      </c>
+          <t>OCR ghi Ø 'DB', Ø8 suy từ kg/m 0.395 — Σ bảng sau sửa khớp tổng bản vẽ — xem PDF tr.31</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr"/>
+      <c r="G29" t="inlineStr"/>
+      <c r="H29" t="inlineStr"/>
       <c r="I29" t="inlineStr"/>
     </row>
     <row r="30">
@@ -35053,21 +35055,21 @@
         <v>27</v>
       </c>
       <c r="B30" t="n">
-        <v>44</v>
+        <v>119</v>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Mố M1</t>
+          <t>Mố M2</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>B1</t>
+          <t>W6(T)</t>
         </is>
       </c>
       <c r="E30" s="11" t="inlineStr">
         <is>
-          <t>OCR ghi Ø 'DB', Ø8 suy từ kg/m 0.395 — Σ bảng sau sửa khớp tổng bản vẽ — xem PDF tr.31</t>
+          <t>BẢN VẼ ghi khối lượng 0 dù dài × SL × kg/m = 51.50 kg — sai trên bản vẽ — xem PDF tr.40</t>
         </is>
       </c>
       <c r="F30" t="inlineStr"/>
@@ -35094,7 +35096,7 @@
       </c>
       <c r="E31" s="11" t="inlineStr">
         <is>
-          <t>BẢN VẼ ghi khối lượng 0 dù dài × SL × kg/m = 51.50 kg — sai trên bản vẽ — xem PDF tr.40</t>
+          <t>Chủ dự án quyết định 11/10/2026: tính các thanh này (bản vẽ ghi 0 kg là sai sót)</t>
         </is>
       </c>
       <c r="F31" t="inlineStr"/>
@@ -35107,7 +35109,7 @@
         <v>29</v>
       </c>
       <c r="B32" t="n">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="C32" t="inlineStr">
         <is>
@@ -35116,12 +35118,12 @@
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>W6(T)</t>
+          <t>W7(T)</t>
         </is>
       </c>
       <c r="E32" s="11" t="inlineStr">
         <is>
-          <t>Chủ dự án quyết định 11/10/2026: tính các thanh này (bản vẽ ghi 0 kg là sai sót)</t>
+          <t>BẢN VẼ ghi khối lượng 0 dù dài × SL × kg/m = 48.84 kg — sai trên bản vẽ — xem PDF tr.40</t>
         </is>
       </c>
       <c r="F32" t="inlineStr"/>
@@ -35148,7 +35150,7 @@
       </c>
       <c r="E33" s="11" t="inlineStr">
         <is>
-          <t>BẢN VẼ ghi khối lượng 0 dù dài × SL × kg/m = 48.84 kg — sai trên bản vẽ — xem PDF tr.40</t>
+          <t>Chủ dự án quyết định 11/10/2026: tính các thanh này (bản vẽ ghi 0 kg là sai sót)</t>
         </is>
       </c>
       <c r="F33" t="inlineStr"/>
@@ -35161,7 +35163,7 @@
         <v>31</v>
       </c>
       <c r="B34" t="n">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="C34" t="inlineStr">
         <is>
@@ -35170,12 +35172,12 @@
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>W7(T)</t>
+          <t>W9(T)</t>
         </is>
       </c>
       <c r="E34" s="11" t="inlineStr">
         <is>
-          <t>Chủ dự án quyết định 11/10/2026: tính các thanh này (bản vẽ ghi 0 kg là sai sót)</t>
+          <t>BẢN VẼ ghi khối lượng 0 dù dài × SL × kg/m = 136.71 kg — sai trên bản vẽ — xem PDF tr.40</t>
         </is>
       </c>
       <c r="F34" t="inlineStr"/>
@@ -35202,7 +35204,7 @@
       </c>
       <c r="E35" s="11" t="inlineStr">
         <is>
-          <t>BẢN VẼ ghi khối lượng 0 dù dài × SL × kg/m = 136.71 kg — sai trên bản vẽ — xem PDF tr.40</t>
+          <t>Chủ dự án quyết định 11/10/2026: tính các thanh này (bản vẽ ghi 0 kg là sai sót)</t>
         </is>
       </c>
       <c r="F35" t="inlineStr"/>
@@ -35215,7 +35217,7 @@
         <v>33</v>
       </c>
       <c r="B36" t="n">
-        <v>122</v>
+        <v>126</v>
       </c>
       <c r="C36" t="inlineStr">
         <is>
@@ -35224,12 +35226,12 @@
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>W9(T)</t>
+          <t>n</t>
         </is>
       </c>
       <c r="E36" s="11" t="inlineStr">
         <is>
-          <t>Chủ dự án quyết định 11/10/2026: tính các thanh này (bản vẽ ghi 0 kg là sai sót)</t>
+          <t>OCR tách chiều dài thành '164' và '0' → 1640 mm; số lượng trống/không đọc được, suy = khối lượng ghi ÷ (dài × kg/m) = 4 — Σ bảng sau sửa khớp tổng bản vẽ — xem PDF tr.40</t>
         </is>
       </c>
       <c r="F36" t="inlineStr"/>
@@ -35242,7 +35244,7 @@
         <v>34</v>
       </c>
       <c r="B37" t="n">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="C37" t="inlineStr">
         <is>
@@ -35251,12 +35253,12 @@
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>n</t>
+          <t>B1</t>
         </is>
       </c>
       <c r="E37" s="11" t="inlineStr">
         <is>
-          <t>OCR tách chiều dài thành '164' và '0' → 1640 mm; số lượng trống/không đọc được, suy = khối lượng ghi ÷ (dài × kg/m) = 4 — Σ bảng sau sửa khớp tổng bản vẽ — xem PDF tr.40</t>
+          <t>OCR tách chiều dài thành '64' và '0' → 640 mm; kg/m không đọc được, lấy 0.395 như các thanh Ø8 khác của bảng; khối lượng 1 cấu kiện không đọc được, lấy từ cột tổng (12.64); số lượng trống/không đọc được, suy = khối lượng ghi ÷ (dài × kg/m) = 50 — Σ bảng sau sửa khớp tổng bản vẽ — xem PDF tr.40</t>
         </is>
       </c>
       <c r="F37" t="inlineStr"/>
@@ -35269,7 +35271,7 @@
         <v>35</v>
       </c>
       <c r="B38" t="n">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="C38" t="inlineStr">
         <is>
@@ -35278,12 +35280,12 @@
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>B1</t>
+          <t>B2</t>
         </is>
       </c>
       <c r="E38" s="11" t="inlineStr">
         <is>
-          <t>OCR tách chiều dài thành '64' và '0' → 640 mm; kg/m không đọc được, lấy 0.395 như các thanh Ø8 khác của bảng; khối lượng 1 cấu kiện không đọc được, lấy từ cột tổng (12.64); số lượng trống/không đọc được, suy = khối lượng ghi ÷ (dài × kg/m) = 50 — Σ bảng sau sửa khớp tổng bản vẽ — xem PDF tr.40</t>
+          <t>OCR tách chiều dài thành '48' và '0' → 480 mm; khối lượng 1 cấu kiện trống, lấy từ cột tổng (12.32) — Σ bảng sau sửa khớp tổng bản vẽ — xem PDF tr.40</t>
         </is>
       </c>
       <c r="F38" t="inlineStr"/>
@@ -35296,7 +35298,7 @@
         <v>36</v>
       </c>
       <c r="B39" t="n">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="C39" t="inlineStr">
         <is>
@@ -35305,12 +35307,12 @@
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>B2</t>
+          <t>T1</t>
         </is>
       </c>
       <c r="E39" s="11" t="inlineStr">
         <is>
-          <t>OCR tách chiều dài thành '48' và '0' → 480 mm; khối lượng 1 cấu kiện trống, lấy từ cột tổng (12.32) — Σ bảng sau sửa khớp tổng bản vẽ — xem PDF tr.40</t>
+          <t>OCR tách chiều dài thành '189' và '0' → 1890 mm; kg/m không đọc được, lấy 1.58 như các thanh Ø16 khác của bảng; khối lượng 1 cấu kiện không đọc được, lấy từ cột tổng (20.90); số lượng trống/không đọc được, suy = khối lượng ghi ÷ (dài × kg/m) = 7 — Σ bảng sau sửa khớp tổng bản vẽ — xem PDF tr.40</t>
         </is>
       </c>
       <c r="F39" t="inlineStr"/>
@@ -35323,7 +35325,7 @@
         <v>37</v>
       </c>
       <c r="B40" t="n">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="C40" t="inlineStr">
         <is>
@@ -35332,12 +35334,12 @@
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>T1</t>
+          <t>T2</t>
         </is>
       </c>
       <c r="E40" s="11" t="inlineStr">
         <is>
-          <t>OCR tách chiều dài thành '189' và '0' → 1890 mm; kg/m không đọc được, lấy 1.58 như các thanh Ø16 khác của bảng; khối lượng 1 cấu kiện không đọc được, lấy từ cột tổng (20.90); số lượng trống/không đọc được, suy = khối lượng ghi ÷ (dài × kg/m) = 7 — Σ bảng sau sửa khớp tổng bản vẽ — xem PDF tr.40</t>
+          <t>OCR tách chiều dài thành '159' và '0' → 1590 mm — Σ bảng sau sửa khớp tổng bản vẽ — xem PDF tr.40</t>
         </is>
       </c>
       <c r="F40" t="inlineStr"/>
@@ -35350,21 +35352,21 @@
         <v>38</v>
       </c>
       <c r="B41" t="n">
-        <v>130</v>
+        <v>134</v>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>Mố M2</t>
+          <t>Trụ T1, T2 (Bệ móng)</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>T2</t>
+          <t>(?)</t>
         </is>
       </c>
       <c r="E41" s="11" t="inlineStr">
         <is>
-          <t>OCR tách chiều dài thành '159' và '0' → 1590 mm — Σ bảng sau sửa khớp tổng bản vẽ — xem PDF tr.40</t>
+          <t>OCR không đọc được ký hiệu thanh (STT 4) — xem PDF tr.44</t>
         </is>
       </c>
       <c r="F41" t="inlineStr"/>
@@ -35377,11 +35379,11 @@
         <v>39</v>
       </c>
       <c r="B42" t="n">
-        <v>134</v>
+        <v>181</v>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>Trụ T1, T2 (Bệ móng)</t>
+          <t>Trụ T1, T2 (Xà mũ trụ)</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
@@ -35391,7 +35393,7 @@
       </c>
       <c r="E42" s="11" t="inlineStr">
         <is>
-          <t>OCR không đọc được ký hiệu thanh (STT 4) — xem PDF tr.44</t>
+          <t>OCR không đọc được ký hiệu thanh (STT 5) — xem PDF tr.51</t>
         </is>
       </c>
       <c r="F42" t="inlineStr"/>
@@ -35404,7 +35406,7 @@
         <v>40</v>
       </c>
       <c r="B43" t="n">
-        <v>181</v>
+        <v>202</v>
       </c>
       <c r="C43" t="inlineStr">
         <is>
@@ -35418,7 +35420,7 @@
       </c>
       <c r="E43" s="11" t="inlineStr">
         <is>
-          <t>OCR không đọc được ký hiệu thanh (STT 5) — xem PDF tr.51</t>
+          <t>OCR không đọc được ký hiệu thanh (STT 5) — xem PDF tr.62</t>
         </is>
       </c>
       <c r="F43" t="inlineStr"/>
@@ -35431,21 +35433,21 @@
         <v>41</v>
       </c>
       <c r="B44" t="n">
-        <v>202</v>
+        <v>233</v>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>Trụ T1, T2 (Xà mũ trụ)</t>
+          <t>Dầm chủ Super-T (15 phiến L=38.2m)</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>(?)</t>
+          <t>G6a</t>
         </is>
       </c>
       <c r="E44" s="11" t="inlineStr">
         <is>
-          <t>OCR không đọc được ký hiệu thanh (STT 5) — xem PDF tr.62</t>
+          <t>OCR đọc SL = 6, phép tính bản vẽ cho 9 (khối lượng ghi ÷ dài ÷ kg/m) — Σ bảng sau sửa khớp tổng bản vẽ — xem PDF tr.88</t>
         </is>
       </c>
       <c r="F44" t="inlineStr"/>
@@ -35458,7 +35460,7 @@
         <v>42</v>
       </c>
       <c r="B45" t="n">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="C45" t="inlineStr">
         <is>
@@ -35467,12 +35469,12 @@
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>G6a</t>
+          <t>G6b</t>
         </is>
       </c>
       <c r="E45" s="11" t="inlineStr">
         <is>
-          <t>OCR đọc SL = 6, phép tính bản vẽ cho 9 (khối lượng ghi ÷ dài ÷ kg/m) — Σ bảng sau sửa khớp tổng bản vẽ — xem PDF tr.88</t>
+          <t>số lượng trống/không đọc được, suy = khối lượng ghi ÷ (dài × kg/m) = 3 — Σ bảng sau sửa khớp tổng bản vẽ — xem PDF tr.88</t>
         </is>
       </c>
       <c r="F45" t="inlineStr"/>
@@ -35485,7 +35487,7 @@
         <v>43</v>
       </c>
       <c r="B46" t="n">
-        <v>234</v>
+        <v>263</v>
       </c>
       <c r="C46" t="inlineStr">
         <is>
@@ -35494,12 +35496,12 @@
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>G6b</t>
+          <t>Thanh neo</t>
         </is>
       </c>
       <c r="E46" s="11" t="inlineStr">
         <is>
-          <t>số lượng trống/không đọc được, suy = khối lượng ghi ÷ (dài × kg/m) = 3 — Σ bảng sau sửa khớp tổng bản vẽ — xem PDF tr.88</t>
+          <t>OCR đọc khối lượng = 217, dài × SL × kg/m = 2.17 — Σ bảng sau sửa khớp tổng bản vẽ — xem PDF tr.91</t>
         </is>
       </c>
       <c r="F46" t="inlineStr"/>
@@ -35512,7 +35514,7 @@
         <v>44</v>
       </c>
       <c r="B47" t="n">
-        <v>263</v>
+        <v>279</v>
       </c>
       <c r="C47" t="inlineStr">
         <is>
@@ -35521,12 +35523,12 @@
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>Thanh neo</t>
+          <t>G6a</t>
         </is>
       </c>
       <c r="E47" s="11" t="inlineStr">
         <is>
-          <t>OCR đọc khối lượng = 217, dài × SL × kg/m = 2.17 — Σ bảng sau sửa khớp tổng bản vẽ — xem PDF tr.91</t>
+          <t>OCR đọc SL = 6, phép tính bản vẽ cho 9 (khối lượng ghi ÷ dài ÷ kg/m) — Σ bảng sau sửa khớp tổng bản vẽ — xem PDF tr.88</t>
         </is>
       </c>
       <c r="F47" t="inlineStr"/>
@@ -35539,7 +35541,7 @@
         <v>45</v>
       </c>
       <c r="B48" t="n">
-        <v>279</v>
+        <v>280</v>
       </c>
       <c r="C48" t="inlineStr">
         <is>
@@ -35548,12 +35550,12 @@
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>G6a</t>
+          <t>G6b</t>
         </is>
       </c>
       <c r="E48" s="11" t="inlineStr">
         <is>
-          <t>OCR đọc SL = 6, phép tính bản vẽ cho 9 (khối lượng ghi ÷ dài ÷ kg/m) — Σ bảng sau sửa khớp tổng bản vẽ — xem PDF tr.88</t>
+          <t>số lượng trống/không đọc được, suy = khối lượng ghi ÷ (dài × kg/m) = 3 — Σ bảng sau sửa khớp tổng bản vẽ — xem PDF tr.88</t>
         </is>
       </c>
       <c r="F48" t="inlineStr"/>
@@ -35566,7 +35568,7 @@
         <v>46</v>
       </c>
       <c r="B49" t="n">
-        <v>280</v>
+        <v>300</v>
       </c>
       <c r="C49" t="inlineStr">
         <is>
@@ -35575,12 +35577,12 @@
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>G6b</t>
+          <t>(?)</t>
         </is>
       </c>
       <c r="E49" s="11" t="inlineStr">
         <is>
-          <t>số lượng trống/không đọc được, suy = khối lượng ghi ÷ (dài × kg/m) = 3 — Σ bảng sau sửa khớp tổng bản vẽ — xem PDF tr.88</t>
+          <t>OCR không đọc được ký hiệu thanh (STT ?) — xem PDF tr.94</t>
         </is>
       </c>
       <c r="F49" t="inlineStr"/>
@@ -35593,7 +35595,7 @@
         <v>47</v>
       </c>
       <c r="B50" t="n">
-        <v>300</v>
+        <v>302</v>
       </c>
       <c r="C50" t="inlineStr">
         <is>
@@ -35602,12 +35604,12 @@
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>(?)</t>
+          <t>G6b</t>
         </is>
       </c>
       <c r="E50" s="11" t="inlineStr">
         <is>
-          <t>OCR không đọc được ký hiệu thanh (STT ?) — xem PDF tr.94</t>
+          <t>số lượng trống/không đọc được, suy = khối lượng ghi ÷ (dài × kg/m) = 3 — Σ bảng sau sửa khớp tổng bản vẽ — xem PDF tr.94</t>
         </is>
       </c>
       <c r="F50" t="inlineStr"/>
@@ -35620,21 +35622,21 @@
         <v>48</v>
       </c>
       <c r="B51" t="n">
-        <v>302</v>
+        <v>312</v>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>Dầm chủ Super-T (15 phiến L=38.2m)</t>
+          <t>Dầm ngang (Diaphragm)</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>G6b</t>
+          <t>A1</t>
         </is>
       </c>
       <c r="E51" s="11" t="inlineStr">
         <is>
-          <t>số lượng trống/không đọc được, suy = khối lượng ghi ÷ (dài × kg/m) = 3 — Σ bảng sau sửa khớp tổng bản vẽ — xem PDF tr.94</t>
+          <t>hệ số 3 suy từ cột tổng (318.54 ÷ 106.18) — xem PDF tr.96</t>
         </is>
       </c>
       <c r="F51" t="inlineStr"/>
@@ -35647,7 +35649,7 @@
         <v>49</v>
       </c>
       <c r="B52" t="n">
-        <v>312</v>
+        <v>313</v>
       </c>
       <c r="C52" t="inlineStr">
         <is>
@@ -35656,12 +35658,12 @@
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>A1</t>
+          <t>A2</t>
         </is>
       </c>
       <c r="E52" s="11" t="inlineStr">
         <is>
-          <t>hệ số 3 suy từ cột tổng (318.54 ÷ 106.18) — xem PDF tr.96</t>
+          <t>hệ số 3 suy từ cột tổng (343.83 ÷ 114.61) — xem PDF tr.96</t>
         </is>
       </c>
       <c r="F52" t="inlineStr"/>
@@ -35674,7 +35676,7 @@
         <v>50</v>
       </c>
       <c r="B53" t="n">
-        <v>313</v>
+        <v>314</v>
       </c>
       <c r="C53" t="inlineStr">
         <is>
@@ -35683,12 +35685,12 @@
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>A2</t>
+          <t>A3</t>
         </is>
       </c>
       <c r="E53" s="11" t="inlineStr">
         <is>
-          <t>hệ số 3 suy từ cột tổng (343.83 ÷ 114.61) — xem PDF tr.96</t>
+          <t>hệ số 3 suy từ cột tổng (737.91 ÷ 245.97) — xem PDF tr.96</t>
         </is>
       </c>
       <c r="F53" t="inlineStr"/>
@@ -35701,7 +35703,7 @@
         <v>51</v>
       </c>
       <c r="B54" t="n">
-        <v>314</v>
+        <v>315</v>
       </c>
       <c r="C54" t="inlineStr">
         <is>
@@ -35710,12 +35712,12 @@
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>A3</t>
+          <t>A4</t>
         </is>
       </c>
       <c r="E54" s="11" t="inlineStr">
         <is>
-          <t>hệ số 3 suy từ cột tổng (737.91 ÷ 245.97) — xem PDF tr.96</t>
+          <t>hệ số 3 suy từ cột tổng (172.92 ÷ 57.64) — xem PDF tr.96</t>
         </is>
       </c>
       <c r="F54" t="inlineStr"/>
@@ -35728,7 +35730,7 @@
         <v>52</v>
       </c>
       <c r="B55" t="n">
-        <v>315</v>
+        <v>316</v>
       </c>
       <c r="C55" t="inlineStr">
         <is>
@@ -35737,12 +35739,12 @@
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>A4</t>
+          <t>A5</t>
         </is>
       </c>
       <c r="E55" s="11" t="inlineStr">
         <is>
-          <t>hệ số 3 suy từ cột tổng (172.92 ÷ 57.64) — xem PDF tr.96</t>
+          <t>hệ số 3 suy từ cột tổng (989.55 ÷ 329.85) — xem PDF tr.96</t>
         </is>
       </c>
       <c r="F55" t="inlineStr"/>
@@ -35755,7 +35757,7 @@
         <v>53</v>
       </c>
       <c r="B56" t="n">
-        <v>316</v>
+        <v>317</v>
       </c>
       <c r="C56" t="inlineStr">
         <is>
@@ -35764,12 +35766,12 @@
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>A5</t>
+          <t>A6</t>
         </is>
       </c>
       <c r="E56" s="11" t="inlineStr">
         <is>
-          <t>hệ số 3 suy từ cột tổng (989.55 ÷ 329.85) — xem PDF tr.96</t>
+          <t>hệ số 3 suy từ cột tổng (200.37 ÷ 66.79) — xem PDF tr.96</t>
         </is>
       </c>
       <c r="F56" t="inlineStr"/>
@@ -35782,21 +35784,21 @@
         <v>54</v>
       </c>
       <c r="B57" t="n">
-        <v>317</v>
+        <v>341</v>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>Dầm ngang (Diaphragm)</t>
+          <t>Bản liên tục nhiệt (Link Slab)</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>A6</t>
+          <t>L1</t>
         </is>
       </c>
       <c r="E57" s="11" t="inlineStr">
         <is>
-          <t>hệ số 3 suy từ cột tổng (200.37 ÷ 66.79) — xem PDF tr.96</t>
+          <t>hệ số 2 suy từ cột tổng (2,837.16 ÷ 1,418.58) — xem PDF tr.112</t>
         </is>
       </c>
       <c r="F57" t="inlineStr"/>
@@ -35823,7 +35825,7 @@
       </c>
       <c r="E58" s="11" t="inlineStr">
         <is>
-          <t>hệ số 2 suy từ cột tổng (2,837.16 ÷ 1,418.58) — xem PDF tr.112</t>
+          <t>OCR ghi Ø 'D1', Ø18 suy từ kg/m 2 — Σ bảng sau sửa khớp tổng bản vẽ — xem PDF tr.112</t>
         </is>
       </c>
       <c r="F58" t="inlineStr"/>
@@ -35836,7 +35838,7 @@
         <v>56</v>
       </c>
       <c r="B59" t="n">
-        <v>341</v>
+        <v>342</v>
       </c>
       <c r="C59" t="inlineStr">
         <is>
@@ -35845,12 +35847,12 @@
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>L1</t>
+          <t>L2</t>
         </is>
       </c>
       <c r="E59" s="11" t="inlineStr">
         <is>
-          <t>OCR ghi Ø 'D1', Ø18 suy từ kg/m 2 — Σ bảng sau sửa khớp tổng bản vẽ — xem PDF tr.112</t>
+          <t>hệ số 2 suy từ cột tổng (5,070.92 ÷ 2,535.46) — xem PDF tr.112</t>
         </is>
       </c>
       <c r="F59" t="inlineStr"/>
@@ -35863,7 +35865,7 @@
         <v>57</v>
       </c>
       <c r="B60" t="n">
-        <v>342</v>
+        <v>343</v>
       </c>
       <c r="C60" t="inlineStr">
         <is>
@@ -35872,12 +35874,12 @@
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>L2</t>
+          <t>L3</t>
         </is>
       </c>
       <c r="E60" s="11" t="inlineStr">
         <is>
-          <t>hệ số 2 suy từ cột tổng (5,070.92 ÷ 2,535.46) — xem PDF tr.112</t>
+          <t>hệ số 2 suy từ cột tổng (102.66 ÷ 51.33) — xem PDF tr.112</t>
         </is>
       </c>
       <c r="F60" t="inlineStr"/>
@@ -35890,7 +35892,7 @@
         <v>58</v>
       </c>
       <c r="B61" t="n">
-        <v>343</v>
+        <v>344</v>
       </c>
       <c r="C61" t="inlineStr">
         <is>
@@ -35899,12 +35901,12 @@
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>L3</t>
+          <t>S4</t>
         </is>
       </c>
       <c r="E61" s="11" t="inlineStr">
         <is>
-          <t>hệ số 2 suy từ cột tổng (102.66 ÷ 51.33) — xem PDF tr.112</t>
+          <t>hệ số 2 suy từ cột tổng (907.20 ÷ 453.60) — xem PDF tr.112</t>
         </is>
       </c>
       <c r="F61" t="inlineStr"/>
@@ -35917,21 +35919,21 @@
         <v>59</v>
       </c>
       <c r="B62" t="n">
-        <v>344</v>
+        <v>360</v>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>Bản liên tục nhiệt (Link Slab)</t>
+          <t>Gờ lan can BTCT</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>S4</t>
+          <t>G1</t>
         </is>
       </c>
       <c r="E62" s="11" t="inlineStr">
         <is>
-          <t>hệ số 2 suy từ cột tổng (907.20 ÷ 453.60) — xem PDF tr.112</t>
+          <t>hệ số 19 suy từ cột tổng (2,581.50 ÷ 135.90) — xem PDF tr.119</t>
         </is>
       </c>
       <c r="F62" t="inlineStr"/>
@@ -35944,7 +35946,7 @@
         <v>60</v>
       </c>
       <c r="B63" t="n">
-        <v>360</v>
+        <v>361</v>
       </c>
       <c r="C63" t="inlineStr">
         <is>
@@ -35953,12 +35955,12 @@
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>G1</t>
+          <t>G2</t>
         </is>
       </c>
       <c r="E63" s="11" t="inlineStr">
         <is>
-          <t>hệ số 19 suy từ cột tổng (2,581.50 ÷ 135.90) — xem PDF tr.119</t>
+          <t>hệ số 19 suy từ cột tổng (4,016.50 ÷ 211.40) — xem PDF tr.119</t>
         </is>
       </c>
       <c r="F63" t="inlineStr"/>
@@ -35971,7 +35973,7 @@
         <v>61</v>
       </c>
       <c r="B64" t="n">
-        <v>361</v>
+        <v>362</v>
       </c>
       <c r="C64" t="inlineStr">
         <is>
@@ -35980,12 +35982,12 @@
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>G2</t>
+          <t>G3</t>
         </is>
       </c>
       <c r="E64" s="11" t="inlineStr">
         <is>
-          <t>hệ số 19 suy từ cột tổng (4,016.50 ÷ 211.40) — xem PDF tr.119</t>
+          <t>hệ số 19 suy từ cột tổng (2,209.40 ÷ 116.30) — xem PDF tr.119</t>
         </is>
       </c>
       <c r="F64" t="inlineStr"/>
@@ -35998,7 +36000,7 @@
         <v>62</v>
       </c>
       <c r="B65" t="n">
-        <v>362</v>
+        <v>363</v>
       </c>
       <c r="C65" t="inlineStr">
         <is>
@@ -36007,12 +36009,12 @@
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>G3</t>
+          <t>G4A</t>
         </is>
       </c>
       <c r="E65" s="11" t="inlineStr">
         <is>
-          <t>hệ số 19 suy từ cột tổng (2,209.40 ÷ 116.30) — xem PDF tr.119</t>
+          <t>khối lượng 1 cấu kiện trống, = dài × SL × kg/m; hệ số 19 = tổng ÷ khối lượng — Σ bảng sau sửa khớp tổng bản vẽ — xem PDF tr.119</t>
         </is>
       </c>
       <c r="F65" t="inlineStr"/>
@@ -36025,7 +36027,7 @@
         <v>63</v>
       </c>
       <c r="B66" t="n">
-        <v>363</v>
+        <v>364</v>
       </c>
       <c r="C66" t="inlineStr">
         <is>
@@ -36034,12 +36036,12 @@
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>G4A</t>
+          <t>G4B</t>
         </is>
       </c>
       <c r="E66" s="11" t="inlineStr">
         <is>
-          <t>khối lượng 1 cấu kiện trống, = dài × SL × kg/m; hệ số 19 = tổng ÷ khối lượng — Σ bảng sau sửa khớp tổng bản vẽ — xem PDF tr.119</t>
+          <t>hệ số 19 suy từ cột tổng (85.10 ÷ dài × SL × kg/m 4.48) — ô số cấu kiện gộp/không đọc được — xem PDF tr.119</t>
         </is>
       </c>
       <c r="F66" t="inlineStr"/>
@@ -36052,7 +36054,7 @@
         <v>64</v>
       </c>
       <c r="B67" t="n">
-        <v>364</v>
+        <v>365</v>
       </c>
       <c r="C67" t="inlineStr">
         <is>
@@ -36061,12 +36063,12 @@
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>G4B</t>
+          <t>G4C</t>
         </is>
       </c>
       <c r="E67" s="11" t="inlineStr">
         <is>
-          <t>hệ số 19 suy từ cột tổng (85.10 ÷ dài × SL × kg/m 4.48) — ô số cấu kiện gộp/không đọc được — xem PDF tr.119</t>
+          <t>hệ số 19 suy từ cột tổng (139.10 ÷ dài × SL × kg/m 7.32) — ô số cấu kiện gộp/không đọc được — xem PDF tr.119</t>
         </is>
       </c>
       <c r="F67" t="inlineStr"/>
@@ -36079,7 +36081,7 @@
         <v>65</v>
       </c>
       <c r="B68" t="n">
-        <v>365</v>
+        <v>372</v>
       </c>
       <c r="C68" t="inlineStr">
         <is>
@@ -36088,12 +36090,12 @@
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>G4C</t>
+          <t>G5</t>
         </is>
       </c>
       <c r="E68" s="11" t="inlineStr">
         <is>
-          <t>hệ số 19 suy từ cột tổng (139.10 ÷ dài × SL × kg/m 7.32) — ô số cấu kiện gộp/không đọc được — xem PDF tr.119</t>
+          <t>hệ số 19 suy từ cột tổng (2,581.50 ÷ 135.90) — xem PDF tr.119</t>
         </is>
       </c>
       <c r="F68" t="inlineStr"/>
@@ -36106,7 +36108,7 @@
         <v>66</v>
       </c>
       <c r="B69" t="n">
-        <v>372</v>
+        <v>373</v>
       </c>
       <c r="C69" t="inlineStr">
         <is>
@@ -36115,12 +36117,12 @@
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>G5</t>
+          <t>G6</t>
         </is>
       </c>
       <c r="E69" s="11" t="inlineStr">
         <is>
-          <t>hệ số 19 suy từ cột tổng (2,581.50 ÷ 135.90) — xem PDF tr.119</t>
+          <t>hệ số 19 suy từ cột tổng (3,898.30 ÷ 205.20) — xem PDF tr.119</t>
         </is>
       </c>
       <c r="F69" t="inlineStr"/>
@@ -36133,7 +36135,7 @@
         <v>67</v>
       </c>
       <c r="B70" t="n">
-        <v>373</v>
+        <v>374</v>
       </c>
       <c r="C70" t="inlineStr">
         <is>
@@ -36142,12 +36144,12 @@
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>G6</t>
+          <t>G7</t>
         </is>
       </c>
       <c r="E70" s="11" t="inlineStr">
         <is>
-          <t>hệ số 19 suy từ cột tổng (3,898.30 ÷ 205.20) — xem PDF tr.119</t>
+          <t>hệ số 19 suy từ cột tổng (1,292.30 ÷ 68.00) — xem PDF tr.119</t>
         </is>
       </c>
       <c r="F70" t="inlineStr"/>
@@ -36160,7 +36162,7 @@
         <v>68</v>
       </c>
       <c r="B71" t="n">
-        <v>374</v>
+        <v>375</v>
       </c>
       <c r="C71" t="inlineStr">
         <is>
@@ -36169,12 +36171,12 @@
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>G7</t>
+          <t>G7A</t>
         </is>
       </c>
       <c r="E71" s="11" t="inlineStr">
         <is>
-          <t>hệ số 19 suy từ cột tổng (1,292.30 ÷ 68.00) — xem PDF tr.119</t>
+          <t>hệ số 19 suy từ cột tổng (2,274.30 ÷ 119.70) — xem PDF tr.119</t>
         </is>
       </c>
       <c r="F71" t="inlineStr"/>
@@ -36187,7 +36189,7 @@
         <v>69</v>
       </c>
       <c r="B72" t="n">
-        <v>375</v>
+        <v>376</v>
       </c>
       <c r="C72" t="inlineStr">
         <is>
@@ -36196,12 +36198,12 @@
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t>G7A</t>
+          <t>G8A</t>
         </is>
       </c>
       <c r="E72" s="11" t="inlineStr">
         <is>
-          <t>hệ số 19 suy từ cột tổng (2,274.30 ÷ 119.70) — xem PDF tr.119</t>
+          <t>hệ số 19 suy từ cột tổng (57.00 ÷ 3.00) — xem PDF tr.119</t>
         </is>
       </c>
       <c r="F72" t="inlineStr"/>
@@ -36214,7 +36216,7 @@
         <v>70</v>
       </c>
       <c r="B73" t="n">
-        <v>376</v>
+        <v>377</v>
       </c>
       <c r="C73" t="inlineStr">
         <is>
@@ -36223,12 +36225,12 @@
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t>G8A</t>
+          <t>G8B</t>
         </is>
       </c>
       <c r="E73" s="11" t="inlineStr">
         <is>
-          <t>hệ số 19 suy từ cột tổng (57.00 ÷ 3.00) — xem PDF tr.119</t>
+          <t>hệ số 19 suy từ cột tổng (67.10 ÷ dài × SL × kg/m 3.53) — ô số cấu kiện gộp/không đọc được — xem PDF tr.119</t>
         </is>
       </c>
       <c r="F73" t="inlineStr"/>
@@ -36241,7 +36243,7 @@
         <v>71</v>
       </c>
       <c r="B74" t="n">
-        <v>377</v>
+        <v>378</v>
       </c>
       <c r="C74" t="inlineStr">
         <is>
@@ -36250,12 +36252,12 @@
       </c>
       <c r="D74" t="inlineStr">
         <is>
-          <t>G8B</t>
+          <t>G8C</t>
         </is>
       </c>
       <c r="E74" s="11" t="inlineStr">
         <is>
-          <t>hệ số 19 suy từ cột tổng (67.10 ÷ dài × SL × kg/m 3.53) — ô số cấu kiện gộp/không đọc được — xem PDF tr.119</t>
+          <t>hệ số 19 suy từ cột tổng (91.50 ÷ dài × SL × kg/m 4.81) — ô số cấu kiện gộp/không đọc được — xem PDF tr.119</t>
         </is>
       </c>
       <c r="F74" t="inlineStr"/>
@@ -36268,7 +36270,7 @@
         <v>72</v>
       </c>
       <c r="B75" t="n">
-        <v>378</v>
+        <v>383</v>
       </c>
       <c r="C75" t="inlineStr">
         <is>
@@ -36277,12 +36279,12 @@
       </c>
       <c r="D75" t="inlineStr">
         <is>
-          <t>G8C</t>
+          <t>G8A</t>
         </is>
       </c>
       <c r="E75" s="11" t="inlineStr">
         <is>
-          <t>hệ số 19 suy từ cột tổng (91.50 ÷ dài × SL × kg/m 4.81) — ô số cấu kiện gộp/không đọc được — xem PDF tr.119</t>
+          <t>OCR đọc SL = 6, phép tính bản vẽ cho 9 (khối lượng ghi ÷ dài ÷ kg/m) — Σ bảng sau sửa khớp tổng bản vẽ — xem PDF tr.119</t>
         </is>
       </c>
       <c r="F75" t="inlineStr"/>
@@ -36295,21 +36297,21 @@
         <v>73</v>
       </c>
       <c r="B76" t="n">
-        <v>383</v>
+        <v>386</v>
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>Gờ lan can BTCT</t>
+          <t>Khe co giãn</t>
         </is>
       </c>
       <c r="D76" t="inlineStr">
         <is>
-          <t>G8A</t>
+          <t>K1</t>
         </is>
       </c>
       <c r="E76" s="11" t="inlineStr">
         <is>
-          <t>OCR đọc SL = 6, phép tính bản vẽ cho 9 (khối lượng ghi ÷ dài ÷ kg/m) — Σ bảng sau sửa khớp tổng bản vẽ — xem PDF tr.119</t>
+          <t>hệ số 2 suy từ cột tổng (586.67 ÷ 293.33) — xem PDF tr.121</t>
         </is>
       </c>
       <c r="F76" t="inlineStr"/>
@@ -36322,7 +36324,7 @@
         <v>74</v>
       </c>
       <c r="B77" t="n">
-        <v>386</v>
+        <v>387</v>
       </c>
       <c r="C77" t="inlineStr">
         <is>
@@ -36331,12 +36333,12 @@
       </c>
       <c r="D77" t="inlineStr">
         <is>
-          <t>K1</t>
+          <t>K2</t>
         </is>
       </c>
       <c r="E77" s="11" t="inlineStr">
         <is>
-          <t>hệ số 2 suy từ cột tổng (586.67 ÷ 293.33) — xem PDF tr.121</t>
+          <t>hệ số 2 suy từ cột tổng (521.99 ÷ 260.99) — xem PDF tr.121</t>
         </is>
       </c>
       <c r="F77" t="inlineStr"/>
@@ -36349,7 +36351,7 @@
         <v>75</v>
       </c>
       <c r="B78" t="n">
-        <v>387</v>
+        <v>388</v>
       </c>
       <c r="C78" t="inlineStr">
         <is>
@@ -36358,12 +36360,12 @@
       </c>
       <c r="D78" t="inlineStr">
         <is>
-          <t>K2</t>
+          <t>K3</t>
         </is>
       </c>
       <c r="E78" s="11" t="inlineStr">
         <is>
-          <t>hệ số 2 suy từ cột tổng (521.99 ÷ 260.99) — xem PDF tr.121</t>
+          <t>hệ số 2 suy từ cột tổng (251.14 ÷ 125.57) — xem PDF tr.121</t>
         </is>
       </c>
       <c r="F78" t="inlineStr"/>
@@ -36371,33 +36373,6 @@
       <c r="H78" t="inlineStr"/>
       <c r="I78" t="inlineStr"/>
     </row>
-    <row r="79">
-      <c r="A79" t="n">
-        <v>76</v>
-      </c>
-      <c r="B79" t="n">
-        <v>388</v>
-      </c>
-      <c r="C79" t="inlineStr">
-        <is>
-          <t>Khe co giãn</t>
-        </is>
-      </c>
-      <c r="D79" t="inlineStr">
-        <is>
-          <t>K3</t>
-        </is>
-      </c>
-      <c r="E79" s="11" t="inlineStr">
-        <is>
-          <t>hệ số 2 suy từ cột tổng (251.14 ÷ 125.57) — xem PDF tr.121</t>
-        </is>
-      </c>
-      <c r="F79" t="inlineStr"/>
-      <c r="G79" t="inlineStr"/>
-      <c r="H79" t="inlineStr"/>
-      <c r="I79" t="inlineStr"/>
-    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>